<commit_message>
Update manual_references.xlsx with new data
</commit_message>
<xml_diff>
--- a/cache/manual_references.xlsx
+++ b/cache/manual_references.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hamidrezabehbood/Documents/GitHub/FReD-data/cache/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103F3E61-A99E-BD4F-8763-5166EDA9D16B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CCF5C8-837C-CD4F-B1CA-2BC239980651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="680" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="831">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="838">
   <si>
     <t>key</t>
   </si>
@@ -4970,6 +4970,27 @@
   </si>
   <si>
     <t>Article 13</t>
+  </si>
+  <si>
+    <t>10.1016/j.im.2015.06.009</t>
+  </si>
+  <si>
+    <t>Hsu, P.-F., Yen, H. R., &amp; Chung, J.-C. (2015). Assessing ERP post-implementation success at the individual level: Revisiting the role of service quality. Information &amp; Management, 52(8), 925–942. https://doi.org/10.1016/j.im.2015.06.009</t>
+  </si>
+  <si>
+    <t>@article{Hsu2015ERP, author={Pei-Fang Hsu and HsiuJu Rebecca Yen and Jung-Ching Chung}, title={Assessing ERP post-implementation success at the individual level: Revisiting the role of service quality}, journal={Information &amp; Management}, year={2015}, volume={52}, number={8}, pages={925--942}, doi={10.1016/j.im.2015.06.009} }</t>
+  </si>
+  <si>
+    <t>Assessing ERP post-implementation success at the individual level: Revisiting the role of service quality</t>
+  </si>
+  <si>
+    <t>Hsu, Pei-Fang; Yen, HsiuJu Rebecca; Chung, Jung-Ching</t>
+  </si>
+  <si>
+    <t>Information &amp; Management</t>
+  </si>
+  <si>
+    <t>925-942</t>
   </si>
 </sst>
 </file>
@@ -5322,7 +5343,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J276"/>
+  <dimension ref="A1:J277"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
@@ -8862,6 +8883,38 @@
         <v>830</v>
       </c>
     </row>
+    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A277" t="s">
+        <v>831</v>
+      </c>
+      <c r="B277" t="s">
+        <v>832</v>
+      </c>
+      <c r="C277" t="s">
+        <v>833</v>
+      </c>
+      <c r="D277" t="s">
+        <v>834</v>
+      </c>
+      <c r="E277" t="s">
+        <v>835</v>
+      </c>
+      <c r="F277" t="s">
+        <v>836</v>
+      </c>
+      <c r="G277">
+        <v>2015</v>
+      </c>
+      <c r="H277">
+        <v>52</v>
+      </c>
+      <c r="I277">
+        <v>8</v>
+      </c>
+      <c r="J277" t="s">
+        <v>837</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update manual_references.xlsx with latest data
</commit_message>
<xml_diff>
--- a/cache/manual_references.xlsx
+++ b/cache/manual_references.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hamidrezabehbood/Documents/GitHub/FReD-data/cache/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hamid\Documents\GitHub\FReD-data\cache\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CCF5C8-837C-CD4F-B1CA-2BC239980651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E9CCA66-2D39-443F-90C4-180339AB495A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4300" yWindow="680" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="841">
   <si>
     <t>key</t>
   </si>
@@ -4992,12 +4992,21 @@
   <si>
     <t>925-942</t>
   </si>
+  <si>
+    <t>https://aisel.aisnet.org/trr/vol7/iss1/3</t>
+  </si>
+  <si>
+    <t>Kumar, M., &amp; Leroy, G. (2021). Factors Affecting Compliance with Alerts in the Context of Healthcare-related Emergencies. AIS Transactions on Replication Research, 7, Article 3. https://doi.org/10.17705/1atrr.00068</t>
+  </si>
+  <si>
+    <t>@article{kumar2021factors, title = {Factors Affecting Compliance with Alerts in the Context of Healthcare-related Emergencies}, author = {Kumar, Manasvi and Leroy, Gondy}, journal = {AIS Transactions on Replication Research}, year = {2021}, volume = {7}, number = {1}, note = {Article 3}, doi = {10.17705/1atrr.00068}, url = {https://aisel.aisnet.org/trr/vol7/iss1/3} }</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5009,6 +5018,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -5034,11 +5050,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5343,10 +5360,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J277"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:SF278"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5378,7 +5395,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -5389,7 +5406,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -5400,7 +5417,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -5411,7 +5428,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -5422,7 +5439,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -5433,7 +5450,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -5444,7 +5461,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -5455,7 +5472,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -5466,7 +5483,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -5477,7 +5494,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>37</v>
       </c>
@@ -5488,7 +5505,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -5499,7 +5516,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -5510,7 +5527,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -5521,7 +5538,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>49</v>
       </c>
@@ -5532,7 +5549,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>52</v>
       </c>
@@ -5543,7 +5560,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>55</v>
       </c>
@@ -5554,7 +5571,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>58</v>
       </c>
@@ -5565,7 +5582,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -5576,7 +5593,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -5587,7 +5604,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>67</v>
       </c>
@@ -5598,7 +5615,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>70</v>
       </c>
@@ -5609,7 +5626,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -5620,7 +5637,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -5631,7 +5648,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -5642,7 +5659,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>82</v>
       </c>
@@ -5650,7 +5667,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>84</v>
       </c>
@@ -5661,7 +5678,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>87</v>
       </c>
@@ -5672,7 +5689,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>90</v>
       </c>
@@ -5683,7 +5700,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>93</v>
       </c>
@@ -5694,7 +5711,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>96</v>
       </c>
@@ -5705,7 +5722,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>99</v>
       </c>
@@ -5716,7 +5733,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>102</v>
       </c>
@@ -5727,7 +5744,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>105</v>
       </c>
@@ -5738,7 +5755,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>108</v>
       </c>
@@ -5749,7 +5766,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>111</v>
       </c>
@@ -5760,7 +5777,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>114</v>
       </c>
@@ -5771,7 +5788,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>117</v>
       </c>
@@ -5782,7 +5799,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>120</v>
       </c>
@@ -5793,7 +5810,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>123</v>
       </c>
@@ -5804,7 +5821,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>126</v>
       </c>
@@ -5815,7 +5832,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>129</v>
       </c>
@@ -5826,7 +5843,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>129</v>
       </c>
@@ -5837,7 +5854,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>129</v>
       </c>
@@ -5848,7 +5865,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>129</v>
       </c>
@@ -5859,7 +5876,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>132</v>
       </c>
@@ -5870,7 +5887,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>135</v>
       </c>
@@ -5881,7 +5898,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>135</v>
       </c>
@@ -5892,7 +5909,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>135</v>
       </c>
@@ -5903,7 +5920,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>138</v>
       </c>
@@ -5914,7 +5931,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>138</v>
       </c>
@@ -5925,7 +5942,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>138</v>
       </c>
@@ -5936,7 +5953,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>141</v>
       </c>
@@ -5947,7 +5964,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>144</v>
       </c>
@@ -5958,7 +5975,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>144</v>
       </c>
@@ -5969,7 +5986,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>144</v>
       </c>
@@ -5980,7 +5997,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>147</v>
       </c>
@@ -5991,7 +6008,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>147</v>
       </c>
@@ -6002,7 +6019,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>147</v>
       </c>
@@ -6013,7 +6030,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>147</v>
       </c>
@@ -6024,7 +6041,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>150</v>
       </c>
@@ -6035,7 +6052,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>153</v>
       </c>
@@ -6046,7 +6063,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>153</v>
       </c>
@@ -6057,7 +6074,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>156</v>
       </c>
@@ -6068,7 +6085,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>156</v>
       </c>
@@ -6079,7 +6096,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>156</v>
       </c>
@@ -6090,7 +6107,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>159</v>
       </c>
@@ -6101,7 +6118,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>159</v>
       </c>
@@ -6112,7 +6129,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>159</v>
       </c>
@@ -6123,7 +6140,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>162</v>
       </c>
@@ -6134,7 +6151,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>162</v>
       </c>
@@ -6145,7 +6162,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>162</v>
       </c>
@@ -6156,7 +6173,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>165</v>
       </c>
@@ -6167,7 +6184,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>168</v>
       </c>
@@ -6178,7 +6195,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>168</v>
       </c>
@@ -6189,7 +6206,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>171</v>
       </c>
@@ -6200,7 +6217,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>171</v>
       </c>
@@ -6211,7 +6228,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>174</v>
       </c>
@@ -6222,7 +6239,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>174</v>
       </c>
@@ -6233,7 +6250,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>174</v>
       </c>
@@ -6244,7 +6261,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>177</v>
       </c>
@@ -6255,7 +6272,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>177</v>
       </c>
@@ -6266,7 +6283,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>177</v>
       </c>
@@ -6277,7 +6294,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>180</v>
       </c>
@@ -6288,7 +6305,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>183</v>
       </c>
@@ -6299,7 +6316,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>186</v>
       </c>
@@ -6310,7 +6327,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>186</v>
       </c>
@@ -6321,7 +6338,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>189</v>
       </c>
@@ -6332,7 +6349,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>192</v>
       </c>
@@ -6343,7 +6360,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>195</v>
       </c>
@@ -6354,7 +6371,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>198</v>
       </c>
@@ -6365,7 +6382,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>201</v>
       </c>
@@ -6376,7 +6393,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>201</v>
       </c>
@@ -6387,7 +6404,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>201</v>
       </c>
@@ -6398,7 +6415,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>201</v>
       </c>
@@ -6409,7 +6426,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>201</v>
       </c>
@@ -6420,7 +6437,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>201</v>
       </c>
@@ -6431,7 +6448,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>201</v>
       </c>
@@ -6442,7 +6459,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>201</v>
       </c>
@@ -6453,7 +6470,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>204</v>
       </c>
@@ -6464,7 +6481,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>207</v>
       </c>
@@ -6475,7 +6492,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>207</v>
       </c>
@@ -6486,7 +6503,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>210</v>
       </c>
@@ -6497,7 +6514,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>213</v>
       </c>
@@ -6508,7 +6525,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>216</v>
       </c>
@@ -6519,7 +6536,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>219</v>
       </c>
@@ -6530,7 +6547,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>219</v>
       </c>
@@ -6541,7 +6558,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>219</v>
       </c>
@@ -6552,7 +6569,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>219</v>
       </c>
@@ -6563,7 +6580,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>222</v>
       </c>
@@ -6574,7 +6591,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>225</v>
       </c>
@@ -6585,7 +6602,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>228</v>
       </c>
@@ -6596,7 +6613,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>231</v>
       </c>
@@ -6607,7 +6624,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>234</v>
       </c>
@@ -6618,7 +6635,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>237</v>
       </c>
@@ -6629,7 +6646,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>240</v>
       </c>
@@ -6640,7 +6657,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>243</v>
       </c>
@@ -6651,7 +6668,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>246</v>
       </c>
@@ -6662,7 +6679,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>249</v>
       </c>
@@ -6673,7 +6690,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>252</v>
       </c>
@@ -6684,7 +6701,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>255</v>
       </c>
@@ -6695,7 +6712,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>258</v>
       </c>
@@ -6706,7 +6723,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>261</v>
       </c>
@@ -6717,7 +6734,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>264</v>
       </c>
@@ -6728,7 +6745,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>267</v>
       </c>
@@ -6739,7 +6756,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>270</v>
       </c>
@@ -6750,7 +6767,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>273</v>
       </c>
@@ -6761,7 +6778,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>276</v>
       </c>
@@ -6772,7 +6789,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>279</v>
       </c>
@@ -6783,7 +6800,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>282</v>
       </c>
@@ -6794,7 +6811,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>285</v>
       </c>
@@ -6805,7 +6822,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>288</v>
       </c>
@@ -6816,7 +6833,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>291</v>
       </c>
@@ -6827,7 +6844,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>294</v>
       </c>
@@ -6838,7 +6855,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>297</v>
       </c>
@@ -6849,7 +6866,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>300</v>
       </c>
@@ -6860,7 +6877,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>303</v>
       </c>
@@ -6871,7 +6888,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>306</v>
       </c>
@@ -6882,7 +6899,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>309</v>
       </c>
@@ -6893,7 +6910,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>312</v>
       </c>
@@ -6904,7 +6921,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>315</v>
       </c>
@@ -6915,7 +6932,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>318</v>
       </c>
@@ -6926,7 +6943,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>321</v>
       </c>
@@ -6937,7 +6954,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>324</v>
       </c>
@@ -6948,7 +6965,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>327</v>
       </c>
@@ -6959,7 +6976,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>330</v>
       </c>
@@ -6970,7 +6987,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>333</v>
       </c>
@@ -6981,7 +6998,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>336</v>
       </c>
@@ -6992,7 +7009,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>339</v>
       </c>
@@ -7003,7 +7020,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>342</v>
       </c>
@@ -7014,7 +7031,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>345</v>
       </c>
@@ -7025,7 +7042,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>348</v>
       </c>
@@ -7036,7 +7053,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>351</v>
       </c>
@@ -7047,7 +7064,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>354</v>
       </c>
@@ -7058,7 +7075,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>357</v>
       </c>
@@ -7069,7 +7086,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>360</v>
       </c>
@@ -7080,7 +7097,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>363</v>
       </c>
@@ -7091,7 +7108,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>366</v>
       </c>
@@ -7102,7 +7119,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>369</v>
       </c>
@@ -7113,7 +7130,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>372</v>
       </c>
@@ -7124,7 +7141,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>375</v>
       </c>
@@ -7135,7 +7152,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>378</v>
       </c>
@@ -7146,7 +7163,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>381</v>
       </c>
@@ -7157,7 +7174,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>384</v>
       </c>
@@ -7168,7 +7185,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>387</v>
       </c>
@@ -7179,7 +7196,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>390</v>
       </c>
@@ -7190,7 +7207,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>393</v>
       </c>
@@ -7201,7 +7218,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>396</v>
       </c>
@@ -7212,7 +7229,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>399</v>
       </c>
@@ -7223,7 +7240,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>402</v>
       </c>
@@ -7234,7 +7251,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>405</v>
       </c>
@@ -7245,7 +7262,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>408</v>
       </c>
@@ -7256,7 +7273,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>411</v>
       </c>
@@ -7276,7 +7293,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>416</v>
       </c>
@@ -7296,7 +7313,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>420</v>
       </c>
@@ -7316,7 +7333,7 @@
         <v>2016</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>424</v>
       </c>
@@ -7345,7 +7362,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>432</v>
       </c>
@@ -7374,7 +7391,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>434</v>
       </c>
@@ -7394,7 +7411,7 @@
         <v>2013</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>439</v>
       </c>
@@ -7414,7 +7431,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>444</v>
       </c>
@@ -7434,7 +7451,7 @@
         <v>2014</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>449</v>
       </c>
@@ -7451,7 +7468,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>453</v>
       </c>
@@ -7462,7 +7479,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>456</v>
       </c>
@@ -7473,7 +7490,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>459</v>
       </c>
@@ -7493,7 +7510,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>464</v>
       </c>
@@ -7513,7 +7530,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>469</v>
       </c>
@@ -7539,7 +7556,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>476</v>
       </c>
@@ -7550,7 +7567,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>479</v>
       </c>
@@ -7561,7 +7578,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>482</v>
       </c>
@@ -7572,7 +7589,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>485</v>
       </c>
@@ -7583,7 +7600,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>488</v>
       </c>
@@ -7594,7 +7611,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
         <v>491</v>
       </c>
@@ -7605,7 +7622,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
         <v>494</v>
       </c>
@@ -7616,7 +7633,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>497</v>
       </c>
@@ -7627,7 +7644,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>500</v>
       </c>
@@ -7638,7 +7655,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>503</v>
       </c>
@@ -7649,7 +7666,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>506</v>
       </c>
@@ -7660,7 +7677,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
         <v>509</v>
       </c>
@@ -7671,7 +7688,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>512</v>
       </c>
@@ -7682,7 +7699,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>515</v>
       </c>
@@ -7693,7 +7710,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>518</v>
       </c>
@@ -7704,7 +7721,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A202" t="s">
         <v>521</v>
       </c>
@@ -7715,7 +7732,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A203" t="s">
         <v>524</v>
       </c>
@@ -7726,7 +7743,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
         <v>527</v>
       </c>
@@ -7737,7 +7754,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
         <v>530</v>
       </c>
@@ -7748,7 +7765,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A206" t="s">
         <v>533</v>
       </c>
@@ -7759,7 +7776,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
         <v>536</v>
       </c>
@@ -7770,7 +7787,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
         <v>539</v>
       </c>
@@ -7781,7 +7798,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
         <v>542</v>
       </c>
@@ -7792,7 +7809,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
         <v>545</v>
       </c>
@@ -7803,7 +7820,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A211" t="s">
         <v>548</v>
       </c>
@@ -7814,7 +7831,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A212" t="s">
         <v>551</v>
       </c>
@@ -7825,7 +7842,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A213" t="s">
         <v>554</v>
       </c>
@@ -7836,7 +7853,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A214" t="s">
         <v>557</v>
       </c>
@@ -7847,7 +7864,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A215" t="s">
         <v>560</v>
       </c>
@@ -7858,7 +7875,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A216" t="s">
         <v>563</v>
       </c>
@@ -7869,7 +7886,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A217" t="s">
         <v>566</v>
       </c>
@@ -7880,7 +7897,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A218" t="s">
         <v>569</v>
       </c>
@@ -7891,7 +7908,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A219" t="s">
         <v>572</v>
       </c>
@@ -7902,7 +7919,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A220" t="s">
         <v>575</v>
       </c>
@@ -7913,7 +7930,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A221" t="s">
         <v>578</v>
       </c>
@@ -7924,7 +7941,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A222" t="s">
         <v>581</v>
       </c>
@@ -7935,7 +7952,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A223" t="s">
         <v>584</v>
       </c>
@@ -7946,7 +7963,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A224" t="s">
         <v>587</v>
       </c>
@@ -7957,7 +7974,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A225" t="s">
         <v>590</v>
       </c>
@@ -7968,7 +7985,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A226" t="s">
         <v>593</v>
       </c>
@@ -7979,7 +7996,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A227" t="s">
         <v>596</v>
       </c>
@@ -7990,7 +8007,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A228" t="s">
         <v>599</v>
       </c>
@@ -8001,7 +8018,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A229" t="s">
         <v>602</v>
       </c>
@@ -8012,7 +8029,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A230" t="s">
         <v>605</v>
       </c>
@@ -8023,7 +8040,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A231" t="s">
         <v>608</v>
       </c>
@@ -8034,7 +8051,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A232" t="s">
         <v>611</v>
       </c>
@@ -8045,7 +8062,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A233" t="s">
         <v>614</v>
       </c>
@@ -8056,7 +8073,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A234" t="s">
         <v>617</v>
       </c>
@@ -8067,7 +8084,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A235" t="s">
         <v>620</v>
       </c>
@@ -8078,7 +8095,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A236" t="s">
         <v>623</v>
       </c>
@@ -8089,7 +8106,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A237" t="s">
         <v>626</v>
       </c>
@@ -8100,7 +8117,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A238" t="s">
         <v>629</v>
       </c>
@@ -8111,7 +8128,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A239" t="s">
         <v>632</v>
       </c>
@@ -8122,7 +8139,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A240" t="s">
         <v>635</v>
       </c>
@@ -8133,7 +8150,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A241" t="s">
         <v>638</v>
       </c>
@@ -8144,7 +8161,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A242" t="s">
         <v>641</v>
       </c>
@@ -8155,7 +8172,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A243" t="s">
         <v>644</v>
       </c>
@@ -8166,7 +8183,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A244" t="s">
         <v>647</v>
       </c>
@@ -8177,7 +8194,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A245" t="s">
         <v>650</v>
       </c>
@@ -8188,7 +8205,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A246" t="s">
         <v>653</v>
       </c>
@@ -8199,7 +8216,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A247" t="s">
         <v>656</v>
       </c>
@@ -8210,7 +8227,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A248" t="s">
         <v>659</v>
       </c>
@@ -8221,7 +8238,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A249" t="s">
         <v>662</v>
       </c>
@@ -8232,7 +8249,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A250" t="s">
         <v>665</v>
       </c>
@@ -8243,7 +8260,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A251" t="s">
         <v>668</v>
       </c>
@@ -8254,7 +8271,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A252" t="s">
         <v>671</v>
       </c>
@@ -8265,7 +8282,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A253" t="s">
         <v>674</v>
       </c>
@@ -8276,7 +8293,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A254" t="s">
         <v>677</v>
       </c>
@@ -8308,7 +8325,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A255" t="s">
         <v>686</v>
       </c>
@@ -8340,7 +8357,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A256" t="s">
         <v>694</v>
       </c>
@@ -8366,7 +8383,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A257" t="s">
         <v>701</v>
       </c>
@@ -8392,7 +8409,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A258" t="s">
         <v>708</v>
       </c>
@@ -8412,7 +8429,7 @@
         <v>1999</v>
       </c>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A259" t="s">
         <v>713</v>
       </c>
@@ -8432,7 +8449,7 @@
         <v>1999</v>
       </c>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A260" t="s">
         <v>718</v>
       </c>
@@ -8464,7 +8481,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A261" t="s">
         <v>725</v>
       </c>
@@ -8487,7 +8504,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A262" t="s">
         <v>731</v>
       </c>
@@ -8510,7 +8527,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A263" t="s">
         <v>736</v>
       </c>
@@ -8530,7 +8547,7 @@
         <v>1880</v>
       </c>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A264" t="s">
         <v>741</v>
       </c>
@@ -8562,7 +8579,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A265" t="s">
         <v>750</v>
       </c>
@@ -8594,7 +8611,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A266" t="s">
         <v>758</v>
       </c>
@@ -8617,7 +8634,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A267" t="s">
         <v>763</v>
       </c>
@@ -8646,7 +8663,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A268" t="s">
         <v>771</v>
       </c>
@@ -8663,7 +8680,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A269" t="s">
         <v>776</v>
       </c>
@@ -8686,7 +8703,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A270" t="s">
         <v>782</v>
       </c>
@@ -8709,7 +8726,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A271" t="s">
         <v>787</v>
       </c>
@@ -8729,7 +8746,7 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A272" t="s">
         <v>792</v>
       </c>
@@ -8755,7 +8772,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A273" t="s">
         <v>799</v>
       </c>
@@ -8787,7 +8804,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A274" t="s">
         <v>807</v>
       </c>
@@ -8819,7 +8836,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A275" t="s">
         <v>815</v>
       </c>
@@ -8851,7 +8868,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A276" t="s">
         <v>824</v>
       </c>
@@ -8883,7 +8900,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:500" x14ac:dyDescent="0.45">
       <c r="A277" t="s">
         <v>831</v>
       </c>
@@ -8914,6 +8931,528 @@
       <c r="J277" t="s">
         <v>837</v>
       </c>
+    </row>
+    <row r="278" spans="1:500" x14ac:dyDescent="0.45">
+      <c r="A278" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="B278" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="C278" s="2" t="s">
+        <v>840</v>
+      </c>
+      <c r="D278" s="2" t="s">
+        <v>810</v>
+      </c>
+      <c r="E278" s="2" t="s">
+        <v>811</v>
+      </c>
+      <c r="F278" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="G278" s="2">
+        <v>2021</v>
+      </c>
+      <c r="H278" s="2">
+        <v>7</v>
+      </c>
+      <c r="I278" s="2">
+        <v>1</v>
+      </c>
+      <c r="J278" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="K278" s="2"/>
+      <c r="L278" s="2"/>
+      <c r="M278" s="2"/>
+      <c r="N278" s="2"/>
+      <c r="O278" s="2"/>
+      <c r="P278" s="2"/>
+      <c r="Q278" s="2"/>
+      <c r="R278" s="2"/>
+      <c r="S278" s="2"/>
+      <c r="T278" s="2"/>
+      <c r="U278" s="2"/>
+      <c r="V278" s="2"/>
+      <c r="W278" s="2"/>
+      <c r="X278" s="2"/>
+      <c r="Y278" s="2"/>
+      <c r="Z278" s="2"/>
+      <c r="AA278" s="2"/>
+      <c r="AB278" s="2"/>
+      <c r="AC278" s="2"/>
+      <c r="AD278" s="2"/>
+      <c r="AE278" s="2"/>
+      <c r="AF278" s="2"/>
+      <c r="AG278" s="2"/>
+      <c r="AH278" s="2"/>
+      <c r="AI278" s="2"/>
+      <c r="AJ278" s="2"/>
+      <c r="AK278" s="2"/>
+      <c r="AL278" s="2"/>
+      <c r="AM278" s="2"/>
+      <c r="AN278" s="2"/>
+      <c r="AO278" s="2"/>
+      <c r="AP278" s="2"/>
+      <c r="AQ278" s="2"/>
+      <c r="AR278" s="2"/>
+      <c r="AS278" s="2"/>
+      <c r="AT278" s="2"/>
+      <c r="AU278" s="2"/>
+      <c r="AV278" s="2"/>
+      <c r="AW278" s="2"/>
+      <c r="AX278" s="2"/>
+      <c r="AY278" s="2"/>
+      <c r="AZ278" s="2"/>
+      <c r="BA278" s="2"/>
+      <c r="BB278" s="2"/>
+      <c r="BC278" s="2"/>
+      <c r="BD278" s="2"/>
+      <c r="BE278" s="2"/>
+      <c r="BF278" s="2"/>
+      <c r="BG278" s="2"/>
+      <c r="BH278" s="2"/>
+      <c r="BI278" s="2"/>
+      <c r="BJ278" s="2"/>
+      <c r="BK278" s="2"/>
+      <c r="BL278" s="2"/>
+      <c r="BM278" s="2"/>
+      <c r="BN278" s="2"/>
+      <c r="BO278" s="2"/>
+      <c r="BP278" s="2"/>
+      <c r="BQ278" s="2"/>
+      <c r="BR278" s="2"/>
+      <c r="BS278" s="2"/>
+      <c r="BT278" s="2"/>
+      <c r="BU278" s="2"/>
+      <c r="BV278" s="2"/>
+      <c r="BW278" s="2"/>
+      <c r="BX278" s="2"/>
+      <c r="BY278" s="2"/>
+      <c r="BZ278" s="2"/>
+      <c r="CA278" s="2"/>
+      <c r="CB278" s="2"/>
+      <c r="CC278" s="2"/>
+      <c r="CD278" s="2"/>
+      <c r="CE278" s="2"/>
+      <c r="CF278" s="2"/>
+      <c r="CG278" s="2"/>
+      <c r="CH278" s="2"/>
+      <c r="CI278" s="2"/>
+      <c r="CJ278" s="2"/>
+      <c r="CK278" s="2"/>
+      <c r="CL278" s="2"/>
+      <c r="CM278" s="2"/>
+      <c r="CN278" s="2"/>
+      <c r="CO278" s="2"/>
+      <c r="CP278" s="2"/>
+      <c r="CQ278" s="2"/>
+      <c r="CR278" s="2"/>
+      <c r="CS278" s="2"/>
+      <c r="CT278" s="2"/>
+      <c r="CU278" s="2"/>
+      <c r="CV278" s="2"/>
+      <c r="CW278" s="2"/>
+      <c r="CX278" s="2"/>
+      <c r="CY278" s="2"/>
+      <c r="CZ278" s="2"/>
+      <c r="DA278" s="2"/>
+      <c r="DB278" s="2"/>
+      <c r="DC278" s="2"/>
+      <c r="DD278" s="2"/>
+      <c r="DE278" s="2"/>
+      <c r="DF278" s="2"/>
+      <c r="DG278" s="2"/>
+      <c r="DH278" s="2"/>
+      <c r="DI278" s="2"/>
+      <c r="DJ278" s="2"/>
+      <c r="DK278" s="2"/>
+      <c r="DL278" s="2"/>
+      <c r="DM278" s="2"/>
+      <c r="DN278" s="2"/>
+      <c r="DO278" s="2"/>
+      <c r="DP278" s="2"/>
+      <c r="DQ278" s="2"/>
+      <c r="DR278" s="2"/>
+      <c r="DS278" s="2"/>
+      <c r="DT278" s="2"/>
+      <c r="DU278" s="2"/>
+      <c r="DV278" s="2"/>
+      <c r="DW278" s="2"/>
+      <c r="DX278" s="2"/>
+      <c r="DY278" s="2"/>
+      <c r="DZ278" s="2"/>
+      <c r="EA278" s="2"/>
+      <c r="EB278" s="2"/>
+      <c r="EC278" s="2"/>
+      <c r="ED278" s="2"/>
+      <c r="EE278" s="2"/>
+      <c r="EF278" s="2"/>
+      <c r="EG278" s="2"/>
+      <c r="EH278" s="2"/>
+      <c r="EI278" s="2"/>
+      <c r="EJ278" s="2"/>
+      <c r="EK278" s="2"/>
+      <c r="EL278" s="2"/>
+      <c r="EM278" s="2"/>
+      <c r="EN278" s="2"/>
+      <c r="EO278" s="2"/>
+      <c r="EP278" s="2"/>
+      <c r="EQ278" s="2"/>
+      <c r="ER278" s="2"/>
+      <c r="ES278" s="2"/>
+      <c r="ET278" s="2"/>
+      <c r="EU278" s="2"/>
+      <c r="EV278" s="2"/>
+      <c r="EW278" s="2"/>
+      <c r="EX278" s="2"/>
+      <c r="EY278" s="2"/>
+      <c r="EZ278" s="2"/>
+      <c r="FA278" s="2"/>
+      <c r="FB278" s="2"/>
+      <c r="FC278" s="2"/>
+      <c r="FD278" s="2"/>
+      <c r="FE278" s="2"/>
+      <c r="FF278" s="2"/>
+      <c r="FG278" s="2"/>
+      <c r="FH278" s="2"/>
+      <c r="FI278" s="2"/>
+      <c r="FJ278" s="2"/>
+      <c r="FK278" s="2"/>
+      <c r="FL278" s="2"/>
+      <c r="FM278" s="2"/>
+      <c r="FN278" s="2"/>
+      <c r="FO278" s="2"/>
+      <c r="FP278" s="2"/>
+      <c r="FQ278" s="2"/>
+      <c r="FR278" s="2"/>
+      <c r="FS278" s="2"/>
+      <c r="FT278" s="2"/>
+      <c r="FU278" s="2"/>
+      <c r="FV278" s="2"/>
+      <c r="FW278" s="2"/>
+      <c r="FX278" s="2"/>
+      <c r="FY278" s="2"/>
+      <c r="FZ278" s="2"/>
+      <c r="GA278" s="2"/>
+      <c r="GB278" s="2"/>
+      <c r="GC278" s="2"/>
+      <c r="GD278" s="2"/>
+      <c r="GE278" s="2"/>
+      <c r="GF278" s="2"/>
+      <c r="GG278" s="2"/>
+      <c r="GH278" s="2"/>
+      <c r="GI278" s="2"/>
+      <c r="GJ278" s="2"/>
+      <c r="GK278" s="2"/>
+      <c r="GL278" s="2"/>
+      <c r="GM278" s="2"/>
+      <c r="GN278" s="2"/>
+      <c r="GO278" s="2"/>
+      <c r="GP278" s="2"/>
+      <c r="GQ278" s="2"/>
+      <c r="GR278" s="2"/>
+      <c r="GS278" s="2"/>
+      <c r="GT278" s="2"/>
+      <c r="GU278" s="2"/>
+      <c r="GV278" s="2"/>
+      <c r="GW278" s="2"/>
+      <c r="GX278" s="2"/>
+      <c r="GY278" s="2"/>
+      <c r="GZ278" s="2"/>
+      <c r="HA278" s="2"/>
+      <c r="HB278" s="2"/>
+      <c r="HC278" s="2"/>
+      <c r="HD278" s="2"/>
+      <c r="HE278" s="2"/>
+      <c r="HF278" s="2"/>
+      <c r="HG278" s="2"/>
+      <c r="HH278" s="2"/>
+      <c r="HI278" s="2"/>
+      <c r="HJ278" s="2"/>
+      <c r="HK278" s="2"/>
+      <c r="HL278" s="2"/>
+      <c r="HM278" s="2"/>
+      <c r="HN278" s="2"/>
+      <c r="HO278" s="2"/>
+      <c r="HP278" s="2"/>
+      <c r="HQ278" s="2"/>
+      <c r="HR278" s="2"/>
+      <c r="HS278" s="2"/>
+      <c r="HT278" s="2"/>
+      <c r="HU278" s="2"/>
+      <c r="HV278" s="2"/>
+      <c r="HW278" s="2"/>
+      <c r="HX278" s="2"/>
+      <c r="HY278" s="2"/>
+      <c r="HZ278" s="2"/>
+      <c r="IA278" s="2"/>
+      <c r="IB278" s="2"/>
+      <c r="IC278" s="2"/>
+      <c r="ID278" s="2"/>
+      <c r="IE278" s="2"/>
+      <c r="IF278" s="2"/>
+      <c r="IG278" s="2"/>
+      <c r="IH278" s="2"/>
+      <c r="II278" s="2"/>
+      <c r="IJ278" s="2"/>
+      <c r="IK278" s="2"/>
+      <c r="IL278" s="2"/>
+      <c r="IM278" s="2"/>
+      <c r="IN278" s="2"/>
+      <c r="IO278" s="2"/>
+      <c r="IP278" s="2"/>
+      <c r="IQ278" s="2"/>
+      <c r="IR278" s="2"/>
+      <c r="IS278" s="2"/>
+      <c r="IT278" s="2"/>
+      <c r="IU278" s="2"/>
+      <c r="IV278" s="2"/>
+      <c r="IW278" s="2"/>
+      <c r="IX278" s="2"/>
+      <c r="IY278" s="2"/>
+      <c r="IZ278" s="2"/>
+      <c r="JA278" s="2"/>
+      <c r="JB278" s="2"/>
+      <c r="JC278" s="2"/>
+      <c r="JD278" s="2"/>
+      <c r="JE278" s="2"/>
+      <c r="JF278" s="2"/>
+      <c r="JG278" s="2"/>
+      <c r="JH278" s="2"/>
+      <c r="JI278" s="2"/>
+      <c r="JJ278" s="2"/>
+      <c r="JK278" s="2"/>
+      <c r="JL278" s="2"/>
+      <c r="JM278" s="2"/>
+      <c r="JN278" s="2"/>
+      <c r="JO278" s="2"/>
+      <c r="JP278" s="2"/>
+      <c r="JQ278" s="2"/>
+      <c r="JR278" s="2"/>
+      <c r="JS278" s="2"/>
+      <c r="JT278" s="2"/>
+      <c r="JU278" s="2"/>
+      <c r="JV278" s="2"/>
+      <c r="JW278" s="2"/>
+      <c r="JX278" s="2"/>
+      <c r="JY278" s="2"/>
+      <c r="JZ278" s="2"/>
+      <c r="KA278" s="2"/>
+      <c r="KB278" s="2"/>
+      <c r="KC278" s="2"/>
+      <c r="KD278" s="2"/>
+      <c r="KE278" s="2"/>
+      <c r="KF278" s="2"/>
+      <c r="KG278" s="2"/>
+      <c r="KH278" s="2"/>
+      <c r="KI278" s="2"/>
+      <c r="KJ278" s="2"/>
+      <c r="KK278" s="2"/>
+      <c r="KL278" s="2"/>
+      <c r="KM278" s="2"/>
+      <c r="KN278" s="2"/>
+      <c r="KO278" s="2"/>
+      <c r="KP278" s="2"/>
+      <c r="KQ278" s="2"/>
+      <c r="KR278" s="2"/>
+      <c r="KS278" s="2"/>
+      <c r="KT278" s="2"/>
+      <c r="KU278" s="2"/>
+      <c r="KV278" s="2"/>
+      <c r="KW278" s="2"/>
+      <c r="KX278" s="2"/>
+      <c r="KY278" s="2"/>
+      <c r="KZ278" s="2"/>
+      <c r="LA278" s="2"/>
+      <c r="LB278" s="2"/>
+      <c r="LC278" s="2"/>
+      <c r="LD278" s="2"/>
+      <c r="LE278" s="2"/>
+      <c r="LF278" s="2"/>
+      <c r="LG278" s="2"/>
+      <c r="LH278" s="2"/>
+      <c r="LI278" s="2"/>
+      <c r="LJ278" s="2"/>
+      <c r="LK278" s="2"/>
+      <c r="LL278" s="2"/>
+      <c r="LM278" s="2"/>
+      <c r="LN278" s="2"/>
+      <c r="LO278" s="2"/>
+      <c r="LP278" s="2"/>
+      <c r="LQ278" s="2"/>
+      <c r="LR278" s="2"/>
+      <c r="LS278" s="2"/>
+      <c r="LT278" s="2"/>
+      <c r="LU278" s="2"/>
+      <c r="LV278" s="2"/>
+      <c r="LW278" s="2"/>
+      <c r="LX278" s="2"/>
+      <c r="LY278" s="2"/>
+      <c r="LZ278" s="2"/>
+      <c r="MA278" s="2"/>
+      <c r="MB278" s="2"/>
+      <c r="MC278" s="2"/>
+      <c r="MD278" s="2"/>
+      <c r="ME278" s="2"/>
+      <c r="MF278" s="2"/>
+      <c r="MG278" s="2"/>
+      <c r="MH278" s="2"/>
+      <c r="MI278" s="2"/>
+      <c r="MJ278" s="2"/>
+      <c r="MK278" s="2"/>
+      <c r="ML278" s="2"/>
+      <c r="MM278" s="2"/>
+      <c r="MN278" s="2"/>
+      <c r="MO278" s="2"/>
+      <c r="MP278" s="2"/>
+      <c r="MQ278" s="2"/>
+      <c r="MR278" s="2"/>
+      <c r="MS278" s="2"/>
+      <c r="MT278" s="2"/>
+      <c r="MU278" s="2"/>
+      <c r="MV278" s="2"/>
+      <c r="MW278" s="2"/>
+      <c r="MX278" s="2"/>
+      <c r="MY278" s="2"/>
+      <c r="MZ278" s="2"/>
+      <c r="NA278" s="2"/>
+      <c r="NB278" s="2"/>
+      <c r="NC278" s="2"/>
+      <c r="ND278" s="2"/>
+      <c r="NE278" s="2"/>
+      <c r="NF278" s="2"/>
+      <c r="NG278" s="2"/>
+      <c r="NH278" s="2"/>
+      <c r="NI278" s="2"/>
+      <c r="NJ278" s="2"/>
+      <c r="NK278" s="2"/>
+      <c r="NL278" s="2"/>
+      <c r="NM278" s="2"/>
+      <c r="NN278" s="2"/>
+      <c r="NO278" s="2"/>
+      <c r="NP278" s="2"/>
+      <c r="NQ278" s="2"/>
+      <c r="NR278" s="2"/>
+      <c r="NS278" s="2"/>
+      <c r="NT278" s="2"/>
+      <c r="NU278" s="2"/>
+      <c r="NV278" s="2"/>
+      <c r="NW278" s="2"/>
+      <c r="NX278" s="2"/>
+      <c r="NY278" s="2"/>
+      <c r="NZ278" s="2"/>
+      <c r="OA278" s="2"/>
+      <c r="OB278" s="2"/>
+      <c r="OC278" s="2"/>
+      <c r="OD278" s="2"/>
+      <c r="OE278" s="2"/>
+      <c r="OF278" s="2"/>
+      <c r="OG278" s="2"/>
+      <c r="OH278" s="2"/>
+      <c r="OI278" s="2"/>
+      <c r="OJ278" s="2"/>
+      <c r="OK278" s="2"/>
+      <c r="OL278" s="2"/>
+      <c r="OM278" s="2"/>
+      <c r="ON278" s="2"/>
+      <c r="OO278" s="2"/>
+      <c r="OP278" s="2"/>
+      <c r="OQ278" s="2"/>
+      <c r="OR278" s="2"/>
+      <c r="OS278" s="2"/>
+      <c r="OT278" s="2"/>
+      <c r="OU278" s="2"/>
+      <c r="OV278" s="2"/>
+      <c r="OW278" s="2"/>
+      <c r="OX278" s="2"/>
+      <c r="OY278" s="2"/>
+      <c r="OZ278" s="2"/>
+      <c r="PA278" s="2"/>
+      <c r="PB278" s="2"/>
+      <c r="PC278" s="2"/>
+      <c r="PD278" s="2"/>
+      <c r="PE278" s="2"/>
+      <c r="PF278" s="2"/>
+      <c r="PG278" s="2"/>
+      <c r="PH278" s="2"/>
+      <c r="PI278" s="2"/>
+      <c r="PJ278" s="2"/>
+      <c r="PK278" s="2"/>
+      <c r="PL278" s="2"/>
+      <c r="PM278" s="2"/>
+      <c r="PN278" s="2"/>
+      <c r="PO278" s="2"/>
+      <c r="PP278" s="2"/>
+      <c r="PQ278" s="2"/>
+      <c r="PR278" s="2"/>
+      <c r="PS278" s="2"/>
+      <c r="PT278" s="2"/>
+      <c r="PU278" s="2"/>
+      <c r="PV278" s="2"/>
+      <c r="PW278" s="2"/>
+      <c r="PX278" s="2"/>
+      <c r="PY278" s="2"/>
+      <c r="PZ278" s="2"/>
+      <c r="QA278" s="2"/>
+      <c r="QB278" s="2"/>
+      <c r="QC278" s="2"/>
+      <c r="QD278" s="2"/>
+      <c r="QE278" s="2"/>
+      <c r="QF278" s="2"/>
+      <c r="QG278" s="2"/>
+      <c r="QH278" s="2"/>
+      <c r="QI278" s="2"/>
+      <c r="QJ278" s="2"/>
+      <c r="QK278" s="2"/>
+      <c r="QL278" s="2"/>
+      <c r="QM278" s="2"/>
+      <c r="QN278" s="2"/>
+      <c r="QO278" s="2"/>
+      <c r="QP278" s="2"/>
+      <c r="QQ278" s="2"/>
+      <c r="QR278" s="2"/>
+      <c r="QS278" s="2"/>
+      <c r="QT278" s="2"/>
+      <c r="QU278" s="2"/>
+      <c r="QV278" s="2"/>
+      <c r="QW278" s="2"/>
+      <c r="QX278" s="2"/>
+      <c r="QY278" s="2"/>
+      <c r="QZ278" s="2"/>
+      <c r="RA278" s="2"/>
+      <c r="RB278" s="2"/>
+      <c r="RC278" s="2"/>
+      <c r="RD278" s="2"/>
+      <c r="RE278" s="2"/>
+      <c r="RF278" s="2"/>
+      <c r="RG278" s="2"/>
+      <c r="RH278" s="2"/>
+      <c r="RI278" s="2"/>
+      <c r="RJ278" s="2"/>
+      <c r="RK278" s="2"/>
+      <c r="RL278" s="2"/>
+      <c r="RM278" s="2"/>
+      <c r="RN278" s="2"/>
+      <c r="RO278" s="2"/>
+      <c r="RP278" s="2"/>
+      <c r="RQ278" s="2"/>
+      <c r="RR278" s="2"/>
+      <c r="RS278" s="2"/>
+      <c r="RT278" s="2"/>
+      <c r="RU278" s="2"/>
+      <c r="RV278" s="2"/>
+      <c r="RW278" s="2"/>
+      <c r="RX278" s="2"/>
+      <c r="RY278" s="2"/>
+      <c r="RZ278" s="2"/>
+      <c r="SA278" s="2"/>
+      <c r="SB278" s="2"/>
+      <c r="SC278" s="2"/>
+      <c r="SD278" s="2"/>
+      <c r="SE278" s="2"/>
+      <c r="SF278" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add manual references for 102 SCORE reproductions with code-name titles
Their OSF records are titled with internal file codes such as
Hansen_JournExpSocPsych_2014_EAa. Replaced with titles naming the
reproduction type and the reproduced paper; author lists repaired
where DataCite recorded SCORE staff as family name [SCORE].

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wa7XA5PkvzBfLidtzNL8RN
</commit_message>
<xml_diff>
--- a/cache/manual_references.xlsx
+++ b/cache/manual_references.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J302"/>
+  <dimension ref="A1:J404"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -10020,6 +10020,3270 @@
         </is>
       </c>
     </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/akubt</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Maier, M., Bartoš, F., &amp; Savi, A. O. (2022). Reproduction (with author data): Hansen &amp; Melzner (2014, Journal of Experimental Social Psychology). OSF. https://doi.org/10.17605/osf.io/akubt</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Hansen &amp; Melzner (2014, Journal of Experimental Social Psychology)</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Maximilian","family":"Maier","sequence":"additional"},{"given":"František","family":"Bartoš","sequence":"additional"},{"given":"Alexander O.","family":"Savi","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/fpuh3</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Weidmann &amp; Callen (2012, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/fpuh3</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Weidmann &amp; Callen (2012, British Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/vndky</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., &amp; … Hanel, P. H. P. (2026). Reproduction (with author data &amp; code): Alves et al. (2018, Psychological Science). OSF. https://doi.org/10.17605/osf.io/vndky</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Alves et al. (2018, Psychological Science)</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>[{"family":"Parsons","given":"E. S.","sequence":"first"},{"family":"Miske","given":"O.","sequence":"additional"},{"family":"Luis","given":"B.","sequence":"additional"},{"family":"Loomas","given":"Z.","sequence":"additional"},{"family":"Fox","given":"N. W.","sequence":"additional"},{"family":"Tyner","given":"A. H.","sequence":"additional"},{"family":"… Hanel","given":"P. H. P.","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/yrh4v</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Christensen et al. (2018, European Journal of Personality). OSF. https://doi.org/10.17605/osf.io/yrh4v</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Christensen et al. (2018, European Journal of Personality)</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/35tgu</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Barreca et al. (2016, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/35tgu</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Barreca et al. (2016, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/zsptj</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Baker &amp; Greene (2011, World Politics). OSF. https://doi.org/10.17605/osf.io/zsptj</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Baker &amp; Greene (2011, World Politics)</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/4y8ja</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): PALER (2013, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/4y8ja</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): PALER (2013, American Political Science Review)</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/nhecx</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): LOUGHRAN et al. (2011, Criminology). OSF. https://doi.org/10.17605/osf.io/nhecx</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): LOUGHRAN et al. (2011, Criminology)</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/qu3p2</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): GROSSMAN &amp; LEWIS (2014, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/qu3p2</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): GROSSMAN &amp; LEWIS (2014, American Political Science Review)</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/3mr7g</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Wang, K. (2022). Reproduction (with author data): Liu et al. (2015, Journal of Marketing). OSF. https://doi.org/10.17605/osf.io/3mr7g</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Liu et al. (2015, Journal of Marketing)</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Ke","family":"Wang","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/axtg4</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Ticku, A. (2022). Reproduction (with author data): Steinmetz et al. (2016, Journal of Personality and Social Psychology). OSF. https://doi.org/10.17605/osf.io/axtg4</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Steinmetz et al. (2016, Journal of Personality and Social Psychology)</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Arunima","family":"Ticku","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/jzfs2</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Ticku, A. (2022). Reproduction (with author data): Brough et al. (2016, Journal of Consumer Research). OSF. https://doi.org/10.17605/osf.io/jzfs2</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Brough et al. (2016, Journal of Consumer Research)</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Arunima","family":"Ticku","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/s57jr</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., McCall, M. C., &amp; Karcher, S. (2022). Reproduction (with author data &amp; code): Li &amp; Zeng (2017, Journal of Experimental Political Science). OSF. https://doi.org/10.17605/osf.io/s57jr</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Li &amp; Zeng (2017, Journal of Experimental Political Science)</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Michael C.","family":"McCall","sequence":"additional"},{"given":"Sebastian","family":"Karcher","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/v9ykq</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Ticku, A. (2022). Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology). OSF. https://doi.org/10.17605/osf.io/v9ykq</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology)</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Arunima","family":"Ticku","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/q5ka2</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Puthillam, A. (2022). Reproduction (with author data &amp; code): LINDQVIST &amp; ÖSTLING (2010, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/q5ka2</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): LINDQVIST &amp; ÖSTLING (2010, American Political Science Review)</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Arathy","family":"Puthillam","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/y47pr</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Martončik, M. (2022). Reproduction (with author data): Ohtsubo et al. (2014, Evolution and Human Behavior). OSF. https://doi.org/10.17605/osf.io/y47pr</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Ohtsubo et al. (2014, Evolution and Human Behavior)</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Marcel","family":"Martončik","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/x9pd3</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Martončik, M. (2022). Reproduction (with author data): Nelson et al. (2009, Journal of Consumer Research). OSF. https://doi.org/10.17605/osf.io/x9pd3</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Nelson et al. (2009, Journal of Consumer Research)</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Marcel","family":"Martončik","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/dcez6</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Urbanska, K. (2022). Reproduction (with author data): Cingranelli et al. (2013, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/dcez6</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Cingranelli et al. (2013, British Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Karolina","family":"Urbanska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/jcbfw</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Bethke, F. (2022). Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/jcbfw</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Felix","family":"Bethke","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/vk2a3</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review). OSF. https://doi.org/10.17605/osf.io/vk2a3</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review)</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Zoran","family":"Pavlović","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/5fc4n</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Bigoni et al. (2015, Econometrica). OSF. https://doi.org/10.17605/osf.io/5fc4n</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Bigoni et al. (2015, Econometrica)</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Zoran","family":"Pavlović","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/hyqpr</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Gerber et al. (2016, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/hyqpr</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Gerber et al. (2016, British Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Zoran","family":"Pavlović","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/57pn2</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Grigoryev, D. (2022). Reproduction (with author data &amp; code): Hertel et al. (2018, Clinical Psychological Science). OSF. https://doi.org/10.17605/osf.io/57pn2</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Hertel et al. (2018, Clinical Psychological Science)</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Dmitry","family":"Grigoryev","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/urfmp</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., … Lou, N., Ph.D. (2026). Reproduction (with author data &amp; code): Wilfahrt (2018, World Politics). OSF. https://doi.org/10.17605/osf.io/urfmp</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Wilfahrt (2018, World Politics)</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>[{"family":"Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., … Lou, N., Ph.D.","given":"","sequence":"first"}]</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/vc8hs</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., Urbanska, K., &amp; Silverstein, P. (2022). Reproduction (with author data): Petersen et al. (2017, Cognition). OSF. https://doi.org/10.17605/osf.io/vc8hs</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Petersen et al. (2017, Cognition)</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Karolina","family":"Urbanska","sequence":"additional"},{"given":"Priya","family":"Silverstein","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/c4ar6</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Evans, T. R. (2022). Reproduction (with author data &amp; code): King &amp; Bryant (2016, Journal of Organizational Behavior). OSF. https://doi.org/10.17605/osf.io/c4ar6</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): King &amp; Bryant (2016, Journal of Organizational Behavior)</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Thomas Rhys","family":"Evans","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/8eqk6</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Sliwka &amp; Werner (2017, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/8eqk6</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Sliwka &amp; Werner (2017, Journal of Labor Economics)</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/3a5u7</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Puthillam, A., &amp; Mehta, N. (2021). Reproduction (with author data &amp; code): Bruner (2017, Experimental Economics). OSF. https://doi.org/10.17605/osf.io/3a5u7</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Bruner (2017, Experimental Economics)</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Arathy","family":"Puthillam","sequence":"additional"},{"given":"Nikita","family":"Mehta","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/u3y9w</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Rovny (2014, World Politics). OSF. https://doi.org/10.17605/osf.io/u3y9w</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Rovny (2014, World Politics)</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Zoran","family":"Pavlović","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/dxmrb</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., Burak, E. G. D., &amp; Loomas, Z. (2021). Reproduction (with author data): Ihme &amp; Tausendpfund (2017, Journal of Experimental Political Science). OSF. https://doi.org/10.17605/osf.io/dxmrb</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Ihme &amp; Tausendpfund (2017, Journal of Experimental Political Science)</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Elif Gizem Demirag","family":"Burak","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/sc87r</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Suchow, J. (2021). Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science). OSF. https://doi.org/10.17605/osf.io/sc87r</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science)</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Jordan","family":"Suchow","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/wnv8y</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Karcher, S., &amp; McCall, M. C. (2022). Reproduction (with author data &amp; code): PIETRYKA &amp; DEBATS (2017, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/wnv8y</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): PIETRYKA &amp; DEBATS (2017, American Political Science Review)</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Sebastian","family":"Karcher","sequence":"additional"},{"given":"Michael C.","family":"McCall","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/5a7qp</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data): Robertson (2015, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/5a7qp</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Robertson (2015, British Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Zoran","family":"Pavlović","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/563d4</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Tagat, A., &amp; Balaji, A. (2022). Reproduction (with author data &amp; code): Angrist &amp; Lavy (2009, American Economic Review). OSF. https://doi.org/10.17605/osf.io/563d4</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Angrist &amp; Lavy (2009, American Economic Review)</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anirudh","family":"Tagat","sequence":"additional"},{"given":"Akshaya","family":"Balaji","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/frc3x</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Urbanska, K. (2022). Reproduction (with author data): Shahar et al. (2016, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/frc3x</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Shahar et al. (2016, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Karolina","family":"Urbanska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/namvy</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/namvy</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/gk6mh</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Kucik &amp; Pelc (2015, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/gk6mh</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Kucik &amp; Pelc (2015, British Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/w8n3s</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Van Dessel, P. (2021). Reproduction (with author data): Axt et al. (2018, Journal of Experimental Social Psychology). OSF. https://doi.org/10.17605/osf.io/w8n3s</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Axt et al. (2018, Journal of Experimental Social Psychology)</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Pieter","family":"Van Dessel","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/gpyu7</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Tagat, A. (2021). Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica). OSF. https://doi.org/10.17605/osf.io/gpyu7</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica)</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anirudh","family":"Tagat","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/sv9tm</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Tagat, A. (2021). Reproduction (with author data &amp; code): McDevitt (2014, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/sv9tm</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): McDevitt (2014, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anirudh","family":"Tagat","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/vh5u6</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlov, Y. G. (2021). Reproduction (with author data): Linkenauger et al. (2009, Psychological Science). OSF. https://doi.org/10.17605/osf.io/vh5u6</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Linkenauger et al. (2009, Psychological Science)</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Yuri G.","family":"Pavlov","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/6mdxr</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Tutor, M. (2022). Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/6mdxr</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics)</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/g2jua</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2021). Reproduction (with author data &amp; code): PICKETT &amp; BAKER (2014, Criminology). OSF. https://doi.org/10.17605/osf.io/g2jua</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): PICKETT &amp; BAKER (2014, Criminology)</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/h2u96</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Peter, N. (2022). Reproduction (with author data &amp; code): Anderson (2011, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/h2u96</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Anderson (2011, American Economic Journal: Applied Economics)</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Noemi","family":"Peter","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/qs827</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2021). Reproduction (with author data &amp; code): Barsbai et al. (2017, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/qs827</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Barsbai et al. (2017, American Economic Journal: Applied Economics)</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/tgkhv</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Andreoni et al. (2017, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/tgkhv</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Andreoni et al. (2017, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/d4p59</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Menaldo (2015, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/d4p59</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Menaldo (2015, American Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/vfyxz</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Fuhrmann &amp; Kreps (2010, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/vfyxz</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Fuhrmann &amp; Kreps (2010, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/ujmvw</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Behrman et al. (2015, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/ujmvw</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Behrman et al. (2015, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/p7tb4</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): McKibben (2013, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/p7tb4</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): McKibben (2013, American Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/ks6ut</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Wilde et al. (2010, American Sociological Review). OSF. https://doi.org/10.17605/osf.io/ks6ut</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Wilde et al. (2010, American Sociological Review)</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/qnmrj</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Fehr et al. (2011, American Economic Review). OSF. https://doi.org/10.17605/osf.io/qnmrj</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Fehr et al. (2011, American Economic Review)</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/5vntp</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Marshall &amp; Fisher (2014, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/5vntp</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Marshall &amp; Fisher (2014, British Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/jp3qb</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Brancati &amp; Snyder (2012, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/jp3qb</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Brancati &amp; Snyder (2012, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/ezx2k</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Wang (2013, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/ezx2k</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Wang (2013, American Economic Journal: Applied Economics)</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/tmg3z</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Jiang (2018, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/tmg3z</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Jiang (2018, American Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/g83kx</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., Tutor, M., &amp; Parsons, E. S. (2020). Reproduction (with author data &amp; code): Surtees et al. (2010, Health Psychology). OSF. https://doi.org/10.17605/osf.io/g83kx</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Surtees et al. (2010, Health Psychology)</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/4fvzq</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Savani et al. (2010, Psychological Science). OSF. https://doi.org/10.17605/osf.io/4fvzq</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Savani et al. (2010, Psychological Science)</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/jhe6q</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Bursztyn &amp; Coffman (2012, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/jhe6q</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Bursztyn &amp; Coffman (2012, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/swkur</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Lacina (2013, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/swkur</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Lacina (2013, American Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/xue5d</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Kehoe &amp; Ruhl (2013, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/xue5d</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Kehoe &amp; Ruhl (2013, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/f3p2m</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Bauer et al. (2015, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/f3p2m</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Bauer et al. (2015, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/xshrn</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Gartzke &amp; Jo (2009, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/xshrn</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Gartzke &amp; Jo (2009, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/wb524</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Miller &amp; Elgün (2010, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/wb524</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Miller &amp; Elgün (2010, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/eqyhz</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., Struhl, M. K., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Liang et al. (2018, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/eqyhz</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Liang et al. (2018, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/adxj2</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Wright &amp; Diehl (2014, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/adxj2</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Wright &amp; Diehl (2014, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/yfvzr</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Evans, T. R. (2020). Reproduction (with author data &amp; code): Hou et al. (2017, Child Development). OSF. https://doi.org/10.17605/osf.io/yfvzr</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Hou et al. (2017, Child Development)</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Thomas Rhys","family":"Evans","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/rpc54</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Wlezien (2016, Comparative Political Studies). OSF. https://doi.org/10.17605/osf.io/rpc54</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Wlezien (2016, Comparative Political Studies)</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/38zs9</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/38zs9</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review)</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/8xyhb</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., Tutor, M., Talbert, E., Parsons, E. S., &amp; Hahn, K. (2020). Reproduction (with author data &amp; code): Beaman et al. (2018, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/8xyhb</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Beaman et al. (2018, Journal of Labor Economics)</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/6e9ka</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Talbert, E., &amp; Errington, T. M. (2020). Reproduction (with author data &amp; code): Turcu &amp; Urbatsch (2014, Comparative Political Studies). OSF. https://doi.org/10.17605/osf.io/6e9ka</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Turcu &amp; Urbatsch (2014, Comparative Political Studies)</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"},{"given":"Timothy M.","family":"Errington","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/fspwc</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Szabelska, A. (2020). Reproduction (with author data &amp; code): Colaresi (2012, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/fspwc</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Colaresi (2012, American Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/5ywth</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Méndez-Chacón, E., Jankowsky, K., Tyner, A. H., Loomas, Z., Miske, O., Luis, B., Fox, N., &amp; Parsons, E. S. (2020). Reproduction (without author data): Baxter et al. (2014, Social Forces). OSF. https://doi.org/10.17605/osf.io/5ywth</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Reproduction (without author data): Baxter et al. (2014, Social Forces)</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>[{"given":"Esteban","family":"Méndez-Chacón","sequence":"first"},{"given":"Kristin","family":"Jankowsky","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/kup8x</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., Struhl, M. K., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Chen &amp; van Ours (2018, Demography). OSF. https://doi.org/10.17605/osf.io/kup8x</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Chen &amp; van Ours (2018, Demography)</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/j6c8g</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Grose et al. (2014, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/j6c8g</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Grose et al. (2014, American Journal of Political Science)</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/anfk6</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Röer, J. P., Miske, O., Fox, N., Loomas, Z., Luis, B., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Ostermann, T., Michalak, J., &amp; Parsons, E. S. (2020). Reproduction (with author data &amp; code): Hurst &amp; Kavanagh (2017, Evolution and Human Behavior). OSF. https://doi.org/10.17605/osf.io/anfk6</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Hurst &amp; Kavanagh (2017, Evolution and Human Behavior)</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>[{"given":"Jan Philipp","family":"Röer","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Thomas","family":"Ostermann","sequence":"additional"},{"given":"Johannes","family":"Michalak","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/7p5tw</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Szabelska, A., Tyner, A. H., Loomas, Z., Miske, O., Luis, B., Fox, N., &amp; Hahn, K. (2020). Reproduction (with author data): Nagengast et al. (2014, Journal of Educational Psychology). OSF. https://doi.org/10.17605/osf.io/7p5tw</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Nagengast et al. (2014, Journal of Educational Psychology)</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>[{"given":"Anna","family":"Szabelska","sequence":"first"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/6ye5m</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Huntington-Klein, N., Tyner, A. H., Loomas, Z., Miske, O., Fox, N., &amp; Luis, B. (2020). Reproduction (without author data): Horowitz (2018, American Sociological Review). OSF. https://doi.org/10.17605/osf.io/6ye5m</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Reproduction (without author data): Horowitz (2018, American Sociological Review)</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>[{"given":"Nick","family":"Huntington-Klein","sequence":"first"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/4axu6</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Cleave et al. (2013, Experimental Economics). OSF. https://doi.org/10.17605/osf.io/4axu6</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Cleave et al. (2013, Experimental Economics)</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/4p892</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Baccara et al. (2014, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/4p892</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Baccara et al. (2014, American Economic Journal: Applied Economics)</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/kzpf8</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Gay, V., Tyner, A. H., Luis, B., &amp; Fox, N. (2020). Reproduction (without author data): Mosimann &amp; Pontusson (2017, World Politics). OSF. https://doi.org/10.17605/osf.io/kzpf8</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Reproduction (without author data): Mosimann &amp; Pontusson (2017, World Politics)</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>[{"given":"Victor","family":"Gay","sequence":"first"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/yh25j</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Lee, J. (2021). Reproduction (with author data &amp; code): Sandra &amp; Otto (2018, Cognition). OSF. https://doi.org/10.17605/osf.io/yh25j</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Sandra &amp; Otto (2018, Cognition)</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Jessica","family":"Lee","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/5vx27</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Chopik, W. J., &amp; Kołczyńska, M. (2021). Reproduction (with author data &amp; code): Nyhan &amp; Reifler (2015, Journal of Experimental Political Science). OSF. https://doi.org/10.17605/osf.io/5vx27</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Nyhan &amp; Reifler (2015, Journal of Experimental Political Science)</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"William J.","family":"Chopik","sequence":"additional"},{"given":"Marta","family":"Kołczyńska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/u8zk5</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Mushtaq, F. (2022). Reproduction (with author data &amp; code): Rich &amp; Gureckis (2018, Journal of Experimental Psychology: General). OSF. https://doi.org/10.17605/osf.io/u8zk5</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Rich &amp; Gureckis (2018, Journal of Experimental Psychology: General)</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Faisal","family":"Mushtaq","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/jfxnt</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Schmidt, K. (2022). Reproduction (with author data): Savani et al. (2010, Psychological Science). OSF. https://doi.org/10.17605/osf.io/jfxnt</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Savani et al. (2010, Psychological Science)</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Kathleen","family":"Schmidt","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/8btme</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Shaki, S., Miske, O., Loomas, Z., Luis, B., Struhl, M. K., Fox, N., Tyner, A. H., Abatayo, A. L., &amp; Hahn, K. (2020). Reproduction (with author data): Rinaldi et al. (2016, Cognition). OSF. https://doi.org/10.17605/osf.io/8btme</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Rinaldi et al. (2016, Cognition)</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>[{"given":"Samuel","family":"Shaki","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/nekdp</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Gereke, J., Field, S., Loomas, Z., Miske, O., Luis, B., Zhang, N., Winter, F., &amp; Kretschmer, D. (2019). Reproduction (without author data): Smith et al. (2016, American Journal of Sociology). OSF. https://doi.org/10.17605/osf.io/nekdp</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Reproduction (without author data): Smith et al. (2016, American Journal of Sociology)</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>[{"given":"Johanna","family":"Gereke","sequence":"first"},{"given":"Samuel","family":"Field","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nan","family":"Zhang","sequence":"additional"},{"given":"Fabian","family":"Winter","sequence":"additional"},{"given":"David","family":"Kretschmer","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/y5uwg</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Chen, J. (., Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Struhl, M. K., Abatayo, A. L., Fox, N., Parsons, E. S., &amp; Hahn, K. (2020). Reproduction (with author data): Goeree et al. (2011, Econometrica). OSF. https://doi.org/10.17605/osf.io/y5uwg</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Goeree et al. (2011, Econometrica)</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>[{"given":"Jingnan (Cecilia)","family":"Chen","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/5k8m4</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Izydorczak, K. (2020). Reproduction (with author data &amp; code): Adida et al. (2016, Comparative Political Studies). OSF. https://doi.org/10.17605/osf.io/5k8m4</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Adida et al. (2016, Comparative Political Studies)</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Kamil","family":"Izydorczak","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/mjb97</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Talbert, E., Parsons, E. S., &amp; Hahn, K. (2020). Reproduction (with author data &amp; code): Altmann et al. (2012, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/mjb97</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Altmann et al. (2012, Journal of Labor Economics)</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/8wf3h</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., Struhl, M. K., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Baillon et al. (2018, Econometrica). OSF. https://doi.org/10.17605/osf.io/8wf3h</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Baillon et al. (2018, Econometrica)</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/6wfmz</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Akcinaroglu (2012, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/6wfmz</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Akcinaroglu (2012, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>https://osf.io/w5eb3</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., &amp; … Silverstein, P. (2026). Reproduction (with author data &amp; code): Luttrell et al. (2016, Journal of Experimental Social Psychology). OSF.</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Luttrell et al. (2016, Journal of Experimental Social Psychology)</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>[{"family":"Parsons","given":"E. S.","sequence":"first"},{"family":"Miske","given":"O.","sequence":"additional"},{"family":"Luis","given":"B.","sequence":"additional"},{"family":"Loomas","given":"Z.","sequence":"additional"},{"family":"Fox","given":"N. W.","sequence":"additional"},{"family":"Tyner","given":"A. H.","sequence":"additional"},{"family":"… Silverstein","given":"P.","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>https://osf.io/tsvz4</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Tyner, A. H., Loomas, Z., Miske, O., Luis, B., Breznau, N., Fox, N. W., &amp; Torma, Z. (2026). Reproduction (without author data): Horvat &amp; Evans (2010, European Sociological Review). OSF.</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Reproduction (without author data): Horvat &amp; Evans (2010, European Sociological Review)</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>[{"family":"Tyner","given":"A. H.","sequence":"first"},{"family":"Loomas","given":"Z.","sequence":"additional"},{"family":"Miske","given":"O.","sequence":"additional"},{"family":"Luis","given":"B.","sequence":"additional"},{"family":"Breznau","given":"N.","sequence":"additional"},{"family":"Fox","given":"N. W.","sequence":"additional"},{"family":"Torma","given":"Z.","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/vufm2</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Sonmez, F., Miske, O., Tyner, A. H., Fox, N., Struhl, M. K., Luis, B., &amp; Abatayo, A. L. (2020). Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology). OSF. https://doi.org/10.17605/osf.io/vufm2</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology)</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>[{"given":"Fatih","family":"Sonmez","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/m4hqw</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Talbert, E., &amp; Soderberg, C. K. (2020). Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review). OSF. https://doi.org/10.17605/osf.io/m4hqw</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review)</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"},{"given":"Courtney K.","family":"Soderberg","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/37jd4</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/37jd4</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy)</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/g9aqj</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science). OSF. https://doi.org/10.17605/osf.io/g9aqj</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science)</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/sv3gb</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica). OSF. https://doi.org/10.17605/osf.io/sv3gb</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica)</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/4n7ef</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/4n7ef</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics)</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melba","family":"Tutor","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/ysncd</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/ysncd</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution)</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/gb46p</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Anafinova, S. (2022). Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/gb46p</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review)</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Saule","family":"Anafinova","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Repair SCORE author names and add BibTeX for generated manual references
Covers the remaining reproductions whose DataCite author records list
staff as family name [SCORE], plus three code-name titles with two-word
surnames missed earlier. BibTeX is now supplied for every generated row
so the exported bibtex_ref_r matches the repaired authors.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wa7XA5PkvzBfLidtzNL8RN
</commit_message>
<xml_diff>
--- a/cache/manual_references.xlsx
+++ b/cache/manual_references.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J404"/>
+  <dimension ref="A1:J424"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -10031,6 +10031,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Maier, M., Bartoš, F., &amp; Savi, A. O. (2022). Reproduction (with author data): Hansen &amp; Melzner (2014, Journal of Experimental Social Psychology). OSF. https://doi.org/10.17605/osf.io/akubt</t>
         </is>
       </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Maier, Maximilian and Bartoš, František and Savi, Alexander O.},
+  title = {Reproduction (with author data): Hansen &amp; Melzner (2014, Journal of Experimental Social Psychology)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/akubt}
+}</t>
+        </is>
+      </c>
       <c r="D303" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Hansen &amp; Melzner (2014, Journal of Experimental Social Psychology)</t>
@@ -10063,6 +10074,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Weidmann &amp; Callen (2012, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/fpuh3</t>
         </is>
       </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Weidmann &amp; Callen (2012, British Journal of Political Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/fpuh3}
+}</t>
+        </is>
+      </c>
       <c r="D304" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Weidmann &amp; Callen (2012, British Journal of Political Science)</t>
@@ -10095,6 +10117,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., &amp; … Hanel, P. H. P. (2026). Reproduction (with author data &amp; code): Alves et al. (2018, Psychological Science). OSF. https://doi.org/10.17605/osf.io/vndky</t>
         </is>
       </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>@article{parsons2026,
+  author = {Parsons, E. S. and Miske, O. and Luis, B. and Loomas, Z. and Fox, N. W. and Tyner, A. H. and … Hanel, P. H. P.},
+  title = {Reproduction (with author data &amp; code): Alves et al. (2018, Psychological Science)},
+  journal = {OSF},
+  year = {2026},
+  doi = {10.17605/osf.io/vndky}
+}</t>
+        </is>
+      </c>
       <c r="D305" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Alves et al. (2018, Psychological Science)</t>
@@ -10127,6 +10160,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Christensen et al. (2018, European Journal of Personality). OSF. https://doi.org/10.17605/osf.io/yrh4v</t>
         </is>
       </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Christensen et al. (2018, European Journal of Personality)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/yrh4v}
+}</t>
+        </is>
+      </c>
       <c r="D306" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Christensen et al. (2018, European Journal of Personality)</t>
@@ -10159,6 +10203,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Barreca et al. (2016, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/35tgu</t>
         </is>
       </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Barreca et al. (2016, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/35tgu}
+}</t>
+        </is>
+      </c>
       <c r="D307" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Barreca et al. (2016, Journal of Political Economy)</t>
@@ -10191,6 +10246,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Baker &amp; Greene (2011, World Politics). OSF. https://doi.org/10.17605/osf.io/zsptj</t>
         </is>
       </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Baker &amp; Greene (2011, World Politics)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/zsptj}
+}</t>
+        </is>
+      </c>
       <c r="D308" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Baker &amp; Greene (2011, World Politics)</t>
@@ -10223,6 +10289,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): PALER (2013, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/4y8ja</t>
         </is>
       </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): PALER (2013, American Political Science Review)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/4y8ja}
+}</t>
+        </is>
+      </c>
       <c r="D309" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): PALER (2013, American Political Science Review)</t>
@@ -10255,6 +10332,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): LOUGHRAN et al. (2011, Criminology). OSF. https://doi.org/10.17605/osf.io/nhecx</t>
         </is>
       </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): LOUGHRAN et al. (2011, Criminology)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/nhecx}
+}</t>
+        </is>
+      </c>
       <c r="D310" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): LOUGHRAN et al. (2011, Criminology)</t>
@@ -10287,6 +10375,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): GROSSMAN &amp; LEWIS (2014, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/qu3p2</t>
         </is>
       </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): GROSSMAN &amp; LEWIS (2014, American Political Science Review)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/qu3p2}
+}</t>
+        </is>
+      </c>
       <c r="D311" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): GROSSMAN &amp; LEWIS (2014, American Political Science Review)</t>
@@ -10319,6 +10418,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Wang, K. (2022). Reproduction (with author data): Liu et al. (2015, Journal of Marketing). OSF. https://doi.org/10.17605/osf.io/3mr7g</t>
         </is>
       </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Wang, Ke},
+  title = {Reproduction (with author data): Liu et al. (2015, Journal of Marketing)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/3mr7g}
+}</t>
+        </is>
+      </c>
       <c r="D312" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Liu et al. (2015, Journal of Marketing)</t>
@@ -10351,6 +10461,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Ticku, A. (2022). Reproduction (with author data): Steinmetz et al. (2016, Journal of Personality and Social Psychology). OSF. https://doi.org/10.17605/osf.io/axtg4</t>
         </is>
       </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Ticku, Arunima},
+  title = {Reproduction (with author data): Steinmetz et al. (2016, Journal of Personality and Social Psychology)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/axtg4}
+}</t>
+        </is>
+      </c>
       <c r="D313" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Steinmetz et al. (2016, Journal of Personality and Social Psychology)</t>
@@ -10383,6 +10504,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Ticku, A. (2022). Reproduction (with author data): Brough et al. (2016, Journal of Consumer Research). OSF. https://doi.org/10.17605/osf.io/jzfs2</t>
         </is>
       </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Ticku, Arunima},
+  title = {Reproduction (with author data): Brough et al. (2016, Journal of Consumer Research)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/jzfs2}
+}</t>
+        </is>
+      </c>
       <c r="D314" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Brough et al. (2016, Journal of Consumer Research)</t>
@@ -10415,6 +10547,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., McCall, M. C., &amp; Karcher, S. (2022). Reproduction (with author data &amp; code): Li &amp; Zeng (2017, Journal of Experimental Political Science). OSF. https://doi.org/10.17605/osf.io/s57jr</t>
         </is>
       </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and McCall, Michael C. and Karcher, Sebastian},
+  title = {Reproduction (with author data &amp; code): Li &amp; Zeng (2017, Journal of Experimental Political Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/s57jr}
+}</t>
+        </is>
+      </c>
       <c r="D315" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Li &amp; Zeng (2017, Journal of Experimental Political Science)</t>
@@ -10447,6 +10590,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Ticku, A. (2022). Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology). OSF. https://doi.org/10.17605/osf.io/v9ykq</t>
         </is>
       </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Ticku, Arunima},
+  title = {Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/v9ykq}
+}</t>
+        </is>
+      </c>
       <c r="D316" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology)</t>
@@ -10479,6 +10633,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Puthillam, A. (2022). Reproduction (with author data &amp; code): LINDQVIST &amp; ÖSTLING (2010, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/q5ka2</t>
         </is>
       </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Puthillam, Arathy},
+  title = {Reproduction (with author data &amp; code): LINDQVIST &amp; ÖSTLING (2010, American Political Science Review)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/q5ka2}
+}</t>
+        </is>
+      </c>
       <c r="D317" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): LINDQVIST &amp; ÖSTLING (2010, American Political Science Review)</t>
@@ -10511,6 +10676,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Martončik, M. (2022). Reproduction (with author data): Ohtsubo et al. (2014, Evolution and Human Behavior). OSF. https://doi.org/10.17605/osf.io/y47pr</t>
         </is>
       </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Martončik, Marcel},
+  title = {Reproduction (with author data): Ohtsubo et al. (2014, Evolution and Human Behavior)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/y47pr}
+}</t>
+        </is>
+      </c>
       <c r="D318" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Ohtsubo et al. (2014, Evolution and Human Behavior)</t>
@@ -10543,6 +10719,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Martončik, M. (2022). Reproduction (with author data): Nelson et al. (2009, Journal of Consumer Research). OSF. https://doi.org/10.17605/osf.io/x9pd3</t>
         </is>
       </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Martončik, Marcel},
+  title = {Reproduction (with author data): Nelson et al. (2009, Journal of Consumer Research)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/x9pd3}
+}</t>
+        </is>
+      </c>
       <c r="D319" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Nelson et al. (2009, Journal of Consumer Research)</t>
@@ -10575,6 +10762,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Urbanska, K. (2022). Reproduction (with author data): Cingranelli et al. (2013, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/dcez6</t>
         </is>
       </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Urbanska, Karolina},
+  title = {Reproduction (with author data): Cingranelli et al. (2013, British Journal of Political Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/dcez6}
+}</t>
+        </is>
+      </c>
       <c r="D320" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Cingranelli et al. (2013, British Journal of Political Science)</t>
@@ -10607,6 +10805,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Bethke, F. (2022). Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/jcbfw</t>
         </is>
       </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Bethke, Felix},
+  title = {Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/jcbfw}
+}</t>
+        </is>
+      </c>
       <c r="D321" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution)</t>
@@ -10639,6 +10848,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review). OSF. https://doi.org/10.17605/osf.io/vk2a3</t>
         </is>
       </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Pavlović, Zoran},
+  title = {Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/vk2a3}
+}</t>
+        </is>
+      </c>
       <c r="D322" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review)</t>
@@ -10671,6 +10891,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Bigoni et al. (2015, Econometrica). OSF. https://doi.org/10.17605/osf.io/5fc4n</t>
         </is>
       </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Pavlović, Zoran},
+  title = {Reproduction (with author data &amp; code): Bigoni et al. (2015, Econometrica)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/5fc4n}
+}</t>
+        </is>
+      </c>
       <c r="D323" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Bigoni et al. (2015, Econometrica)</t>
@@ -10703,6 +10934,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Gerber et al. (2016, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/hyqpr</t>
         </is>
       </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Pavlović, Zoran},
+  title = {Reproduction (with author data &amp; code): Gerber et al. (2016, British Journal of Political Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/hyqpr}
+}</t>
+        </is>
+      </c>
       <c r="D324" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Gerber et al. (2016, British Journal of Political Science)</t>
@@ -10735,6 +10977,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Grigoryev, D. (2022). Reproduction (with author data &amp; code): Hertel et al. (2018, Clinical Psychological Science). OSF. https://doi.org/10.17605/osf.io/57pn2</t>
         </is>
       </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Grigoryev, Dmitry},
+  title = {Reproduction (with author data &amp; code): Hertel et al. (2018, Clinical Psychological Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/57pn2}
+}</t>
+        </is>
+      </c>
       <c r="D325" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Hertel et al. (2018, Clinical Psychological Science)</t>
@@ -10767,6 +11020,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., … Lou, N., Ph.D. (2026). Reproduction (with author data &amp; code): Wilfahrt (2018, World Politics). OSF. https://doi.org/10.17605/osf.io/urfmp</t>
         </is>
       </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>@article{parsonsesmiskeoluisbloomaszfoxnwtynerahlounphd2026,
+  author = {Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., … Lou, N., Ph.D.},
+  title = {Reproduction (with author data &amp; code): Wilfahrt (2018, World Politics)},
+  journal = {OSF},
+  year = {2026},
+  doi = {10.17605/osf.io/urfmp}
+}</t>
+        </is>
+      </c>
       <c r="D326" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Wilfahrt (2018, World Politics)</t>
@@ -10799,6 +11063,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., Urbanska, K., &amp; Silverstein, P. (2022). Reproduction (with author data): Petersen et al. (2017, Cognition). OSF. https://doi.org/10.17605/osf.io/vc8hs</t>
         </is>
       </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Urbanska, Karolina and Silverstein, Priya},
+  title = {Reproduction (with author data): Petersen et al. (2017, Cognition)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/vc8hs}
+}</t>
+        </is>
+      </c>
       <c r="D327" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Petersen et al. (2017, Cognition)</t>
@@ -10831,6 +11106,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Evans, T. R. (2022). Reproduction (with author data &amp; code): King &amp; Bryant (2016, Journal of Organizational Behavior). OSF. https://doi.org/10.17605/osf.io/c4ar6</t>
         </is>
       </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Evans, Thomas Rhys},
+  title = {Reproduction (with author data &amp; code): King &amp; Bryant (2016, Journal of Organizational Behavior)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/c4ar6}
+}</t>
+        </is>
+      </c>
       <c r="D328" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): King &amp; Bryant (2016, Journal of Organizational Behavior)</t>
@@ -10863,6 +11149,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Sliwka &amp; Werner (2017, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/8eqk6</t>
         </is>
       </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Sliwka &amp; Werner (2017, Journal of Labor Economics)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/8eqk6}
+}</t>
+        </is>
+      </c>
       <c r="D329" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Sliwka &amp; Werner (2017, Journal of Labor Economics)</t>
@@ -10895,6 +11192,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Puthillam, A., &amp; Mehta, N. (2021). Reproduction (with author data &amp; code): Bruner (2017, Experimental Economics). OSF. https://doi.org/10.17605/osf.io/3a5u7</t>
         </is>
       </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Puthillam, Arathy and Mehta, Nikita},
+  title = {Reproduction (with author data &amp; code): Bruner (2017, Experimental Economics)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/3a5u7}
+}</t>
+        </is>
+      </c>
       <c r="D330" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Bruner (2017, Experimental Economics)</t>
@@ -10927,6 +11235,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data &amp; code): Rovny (2014, World Politics). OSF. https://doi.org/10.17605/osf.io/u3y9w</t>
         </is>
       </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Pavlović, Zoran},
+  title = {Reproduction (with author data &amp; code): Rovny (2014, World Politics)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/u3y9w}
+}</t>
+        </is>
+      </c>
       <c r="D331" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Rovny (2014, World Politics)</t>
@@ -10959,6 +11278,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., Burak, E. G. D., &amp; Loomas, Z. (2021). Reproduction (with author data): Ihme &amp; Tausendpfund (2017, Journal of Experimental Political Science). OSF. https://doi.org/10.17605/osf.io/dxmrb</t>
         </is>
       </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Burak, Elif Gizem Demirag and Loomas, Zachary},
+  title = {Reproduction (with author data): Ihme &amp; Tausendpfund (2017, Journal of Experimental Political Science)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/dxmrb}
+}</t>
+        </is>
+      </c>
       <c r="D332" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Ihme &amp; Tausendpfund (2017, Journal of Experimental Political Science)</t>
@@ -10991,6 +11321,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Suchow, J. (2021). Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science). OSF. https://doi.org/10.17605/osf.io/sc87r</t>
         </is>
       </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Suchow, Jordan},
+  title = {Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/sc87r}
+}</t>
+        </is>
+      </c>
       <c r="D333" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science)</t>
@@ -11023,6 +11364,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Karcher, S., &amp; McCall, M. C. (2022). Reproduction (with author data &amp; code): PIETRYKA &amp; DEBATS (2017, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/wnv8y</t>
         </is>
       </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Karcher, Sebastian and McCall, Michael C.},
+  title = {Reproduction (with author data &amp; code): PIETRYKA &amp; DEBATS (2017, American Political Science Review)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/wnv8y}
+}</t>
+        </is>
+      </c>
       <c r="D334" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): PIETRYKA &amp; DEBATS (2017, American Political Science Review)</t>
@@ -11055,6 +11407,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlović, Z. (2022). Reproduction (with author data): Robertson (2015, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/5a7qp</t>
         </is>
       </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Pavlović, Zoran},
+  title = {Reproduction (with author data): Robertson (2015, British Journal of Political Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/5a7qp}
+}</t>
+        </is>
+      </c>
       <c r="D335" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Robertson (2015, British Journal of Political Science)</t>
@@ -11087,6 +11450,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Tagat, A., &amp; Balaji, A. (2022). Reproduction (with author data &amp; code): Angrist &amp; Lavy (2009, American Economic Review). OSF. https://doi.org/10.17605/osf.io/563d4</t>
         </is>
       </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Tagat, Anirudh and Balaji, Akshaya},
+  title = {Reproduction (with author data &amp; code): Angrist &amp; Lavy (2009, American Economic Review)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/563d4}
+}</t>
+        </is>
+      </c>
       <c r="D336" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Angrist &amp; Lavy (2009, American Economic Review)</t>
@@ -11119,6 +11493,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Urbanska, K. (2022). Reproduction (with author data): Shahar et al. (2016, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/frc3x</t>
         </is>
       </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Urbanska, Karolina},
+  title = {Reproduction (with author data): Shahar et al. (2016, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/frc3x}
+}</t>
+        </is>
+      </c>
       <c r="D337" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Shahar et al. (2016, Journal of Conflict Resolution)</t>
@@ -11151,6 +11536,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/namvy</t>
         </is>
       </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/namvy}
+}</t>
+        </is>
+      </c>
       <c r="D338" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy)</t>
@@ -11183,6 +11579,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): Kucik &amp; Pelc (2015, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/gk6mh</t>
         </is>
       </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Kucik &amp; Pelc (2015, British Journal of Political Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/gk6mh}
+}</t>
+        </is>
+      </c>
       <c r="D339" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Kucik &amp; Pelc (2015, British Journal of Political Science)</t>
@@ -11215,6 +11622,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Van Dessel, P. (2021). Reproduction (with author data): Axt et al. (2018, Journal of Experimental Social Psychology). OSF. https://doi.org/10.17605/osf.io/w8n3s</t>
         </is>
       </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Van Dessel, Pieter},
+  title = {Reproduction (with author data): Axt et al. (2018, Journal of Experimental Social Psychology)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/w8n3s}
+}</t>
+        </is>
+      </c>
       <c r="D340" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Axt et al. (2018, Journal of Experimental Social Psychology)</t>
@@ -11247,6 +11665,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Tagat, A. (2021). Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica). OSF. https://doi.org/10.17605/osf.io/gpyu7</t>
         </is>
       </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Tagat, Anirudh},
+  title = {Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/gpyu7}
+}</t>
+        </is>
+      </c>
       <c r="D341" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica)</t>
@@ -11279,6 +11708,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Tagat, A. (2021). Reproduction (with author data &amp; code): McDevitt (2014, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/sv9tm</t>
         </is>
       </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Tagat, Anirudh},
+  title = {Reproduction (with author data &amp; code): McDevitt (2014, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/sv9tm}
+}</t>
+        </is>
+      </c>
       <c r="D342" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): McDevitt (2014, Journal of Political Economy)</t>
@@ -11311,6 +11751,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Pavlov, Y. G. (2021). Reproduction (with author data): Linkenauger et al. (2009, Psychological Science). OSF. https://doi.org/10.17605/osf.io/vh5u6</t>
         </is>
       </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Pavlov, Yuri G.},
+  title = {Reproduction (with author data): Linkenauger et al. (2009, Psychological Science)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/vh5u6}
+}</t>
+        </is>
+      </c>
       <c r="D343" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Linkenauger et al. (2009, Psychological Science)</t>
@@ -11343,6 +11794,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Tutor, M. (2022). Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/6mdxr</t>
         </is>
       </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/6mdxr}
+}</t>
+        </is>
+      </c>
       <c r="D344" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics)</t>
@@ -11375,6 +11837,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2021). Reproduction (with author data &amp; code): PICKETT &amp; BAKER (2014, Criminology). OSF. https://doi.org/10.17605/osf.io/g2jua</t>
         </is>
       </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): PICKETT &amp; BAKER (2014, Criminology)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/g2jua}
+}</t>
+        </is>
+      </c>
       <c r="D345" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): PICKETT &amp; BAKER (2014, Criminology)</t>
@@ -11407,6 +11880,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Peter, N. (2022). Reproduction (with author data &amp; code): Anderson (2011, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/h2u96</t>
         </is>
       </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Peter, Noemi},
+  title = {Reproduction (with author data &amp; code): Anderson (2011, American Economic Journal: Applied Economics)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/h2u96}
+}</t>
+        </is>
+      </c>
       <c r="D346" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Anderson (2011, American Economic Journal: Applied Economics)</t>
@@ -11439,6 +11923,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2021). Reproduction (with author data &amp; code): Barsbai et al. (2017, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/qs827</t>
         </is>
       </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Barsbai et al. (2017, American Economic Journal: Applied Economics)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/qs827}
+}</t>
+        </is>
+      </c>
       <c r="D347" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Barsbai et al. (2017, American Economic Journal: Applied Economics)</t>
@@ -11471,6 +11966,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Andreoni et al. (2017, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/tgkhv</t>
         </is>
       </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Andreoni et al. (2017, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/tgkhv}
+}</t>
+        </is>
+      </c>
       <c r="D348" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Andreoni et al. (2017, Journal of Political Economy)</t>
@@ -11503,6 +12009,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Menaldo (2015, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/d4p59</t>
         </is>
       </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Menaldo (2015, American Journal of Political Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/d4p59}
+}</t>
+        </is>
+      </c>
       <c r="D349" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Menaldo (2015, American Journal of Political Science)</t>
@@ -11535,6 +12052,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Fuhrmann &amp; Kreps (2010, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/vfyxz</t>
         </is>
       </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Fuhrmann &amp; Kreps (2010, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/vfyxz}
+}</t>
+        </is>
+      </c>
       <c r="D350" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Fuhrmann &amp; Kreps (2010, Journal of Conflict Resolution)</t>
@@ -11567,6 +12095,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Behrman et al. (2015, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/ujmvw</t>
         </is>
       </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Behrman et al. (2015, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/ujmvw}
+}</t>
+        </is>
+      </c>
       <c r="D351" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Behrman et al. (2015, Journal of Political Economy)</t>
@@ -11599,6 +12138,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): McKibben (2013, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/p7tb4</t>
         </is>
       </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): McKibben (2013, American Journal of Political Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/p7tb4}
+}</t>
+        </is>
+      </c>
       <c r="D352" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): McKibben (2013, American Journal of Political Science)</t>
@@ -11631,6 +12181,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Wilde et al. (2010, American Sociological Review). OSF. https://doi.org/10.17605/osf.io/ks6ut</t>
         </is>
       </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Wilde et al. (2010, American Sociological Review)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/ks6ut}
+}</t>
+        </is>
+      </c>
       <c r="D353" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Wilde et al. (2010, American Sociological Review)</t>
@@ -11663,6 +12224,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Fehr et al. (2011, American Economic Review). OSF. https://doi.org/10.17605/osf.io/qnmrj</t>
         </is>
       </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Fehr et al. (2011, American Economic Review)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/qnmrj}
+}</t>
+        </is>
+      </c>
       <c r="D354" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Fehr et al. (2011, American Economic Review)</t>
@@ -11695,6 +12267,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Marshall &amp; Fisher (2014, British Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/5vntp</t>
         </is>
       </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Marshall &amp; Fisher (2014, British Journal of Political Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/5vntp}
+}</t>
+        </is>
+      </c>
       <c r="D355" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Marshall &amp; Fisher (2014, British Journal of Political Science)</t>
@@ -11727,6 +12310,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Brancati &amp; Snyder (2012, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/jp3qb</t>
         </is>
       </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Brancati &amp; Snyder (2012, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/jp3qb}
+}</t>
+        </is>
+      </c>
       <c r="D356" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Brancati &amp; Snyder (2012, Journal of Conflict Resolution)</t>
@@ -11759,6 +12353,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Wang (2013, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/ezx2k</t>
         </is>
       </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Wang (2013, American Economic Journal: Applied Economics)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/ezx2k}
+}</t>
+        </is>
+      </c>
       <c r="D357" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Wang (2013, American Economic Journal: Applied Economics)</t>
@@ -11791,6 +12396,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Jiang (2018, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/tmg3z</t>
         </is>
       </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Tyner, Andrew H. and Fox, Nicholas and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Jiang (2018, American Journal of Political Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/tmg3z}
+}</t>
+        </is>
+      </c>
       <c r="D358" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Jiang (2018, American Journal of Political Science)</t>
@@ -11823,6 +12439,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., Tutor, M., &amp; Parsons, E. S. (2020). Reproduction (with author data &amp; code): Surtees et al. (2010, Health Psychology). OSF. https://doi.org/10.17605/osf.io/g83kx</t>
         </is>
       </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba and Parsons, Elan Simon},
+  title = {Reproduction (with author data &amp; code): Surtees et al. (2010, Health Psychology)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/g83kx}
+}</t>
+        </is>
+      </c>
       <c r="D359" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Surtees et al. (2010, Health Psychology)</t>
@@ -11855,6 +12482,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Savani et al. (2010, Psychological Science). OSF. https://doi.org/10.17605/osf.io/4fvzq</t>
         </is>
       </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Savani et al. (2010, Psychological Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/4fvzq}
+}</t>
+        </is>
+      </c>
       <c r="D360" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Savani et al. (2010, Psychological Science)</t>
@@ -11887,6 +12525,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Bursztyn &amp; Coffman (2012, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/jhe6q</t>
         </is>
       </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Bursztyn &amp; Coffman (2012, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/jhe6q}
+}</t>
+        </is>
+      </c>
       <c r="D361" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Bursztyn &amp; Coffman (2012, Journal of Political Economy)</t>
@@ -11919,6 +12568,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Lacina (2013, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/swkur</t>
         </is>
       </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Lacina (2013, American Journal of Political Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/swkur}
+}</t>
+        </is>
+      </c>
       <c r="D362" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Lacina (2013, American Journal of Political Science)</t>
@@ -11951,6 +12611,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Kehoe &amp; Ruhl (2013, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/xue5d</t>
         </is>
       </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Kehoe &amp; Ruhl (2013, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/xue5d}
+}</t>
+        </is>
+      </c>
       <c r="D363" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Kehoe &amp; Ruhl (2013, Journal of Political Economy)</t>
@@ -11983,6 +12654,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Bauer et al. (2015, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/f3p2m</t>
         </is>
       </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Bauer et al. (2015, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/f3p2m}
+}</t>
+        </is>
+      </c>
       <c r="D364" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Bauer et al. (2015, Journal of Conflict Resolution)</t>
@@ -12015,6 +12697,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Gartzke &amp; Jo (2009, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/xshrn</t>
         </is>
       </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Gartzke &amp; Jo (2009, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/xshrn}
+}</t>
+        </is>
+      </c>
       <c r="D365" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Gartzke &amp; Jo (2009, Journal of Conflict Resolution)</t>
@@ -12047,6 +12740,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Miller &amp; Elgün (2010, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/wb524</t>
         </is>
       </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Miller &amp; Elgün (2010, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/wb524}
+}</t>
+        </is>
+      </c>
       <c r="D366" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Miller &amp; Elgün (2010, Journal of Conflict Resolution)</t>
@@ -12079,6 +12783,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., Struhl, M. K., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Liang et al. (2018, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/eqyhz</t>
         </is>
       </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Tyner, Andrew H. and Fox, Nicholas and Struhl, Melissa Kline and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Liang et al. (2018, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/eqyhz}
+}</t>
+        </is>
+      </c>
       <c r="D367" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Liang et al. (2018, Journal of Political Economy)</t>
@@ -12111,6 +12826,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Wright &amp; Diehl (2014, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/adxj2</t>
         </is>
       </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Wright &amp; Diehl (2014, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/adxj2}
+}</t>
+        </is>
+      </c>
       <c r="D368" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Wright &amp; Diehl (2014, Journal of Conflict Resolution)</t>
@@ -12143,6 +12869,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Evans, T. R. (2020). Reproduction (with author data &amp; code): Hou et al. (2017, Child Development). OSF. https://doi.org/10.17605/osf.io/yfvzr</t>
         </is>
       </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Evans, Thomas Rhys},
+  title = {Reproduction (with author data &amp; code): Hou et al. (2017, Child Development)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/yfvzr}
+}</t>
+        </is>
+      </c>
       <c r="D369" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Hou et al. (2017, Child Development)</t>
@@ -12175,6 +12912,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Wlezien (2016, Comparative Political Studies). OSF. https://doi.org/10.17605/osf.io/rpc54</t>
         </is>
       </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Wlezien (2016, Comparative Political Studies)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/rpc54}
+}</t>
+        </is>
+      </c>
       <c r="D370" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Wlezien (2016, Comparative Political Studies)</t>
@@ -12207,6 +12955,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/38zs9</t>
         </is>
       </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/38zs9}
+}</t>
+        </is>
+      </c>
       <c r="D371" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review)</t>
@@ -12239,6 +12998,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., Tutor, M., Talbert, E., Parsons, E. S., &amp; Hahn, K. (2020). Reproduction (with author data &amp; code): Beaman et al. (2018, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/8xyhb</t>
         </is>
       </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba and Talbert, Eli and Parsons, Elan Simon and Hahn, Krystal},
+  title = {Reproduction (with author data &amp; code): Beaman et al. (2018, Journal of Labor Economics)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/8xyhb}
+}</t>
+        </is>
+      </c>
       <c r="D372" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Beaman et al. (2018, Journal of Labor Economics)</t>
@@ -12271,6 +13041,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Talbert, E., &amp; Errington, T. M. (2020). Reproduction (with author data &amp; code): Turcu &amp; Urbatsch (2014, Comparative Political Studies). OSF. https://doi.org/10.17605/osf.io/6e9ka</t>
         </is>
       </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Talbert, Eli and Errington, Timothy M.},
+  title = {Reproduction (with author data &amp; code): Turcu &amp; Urbatsch (2014, Comparative Political Studies)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/6e9ka}
+}</t>
+        </is>
+      </c>
       <c r="D373" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Turcu &amp; Urbatsch (2014, Comparative Political Studies)</t>
@@ -12303,6 +13084,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Szabelska, A. (2020). Reproduction (with author data &amp; code): Colaresi (2012, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/fspwc</t>
         </is>
       </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): Colaresi (2012, American Journal of Political Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/fspwc}
+}</t>
+        </is>
+      </c>
       <c r="D374" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Colaresi (2012, American Journal of Political Science)</t>
@@ -12335,6 +13127,17 @@
           <t>Méndez-Chacón, E., Jankowsky, K., Tyner, A. H., Loomas, Z., Miske, O., Luis, B., Fox, N., &amp; Parsons, E. S. (2020). Reproduction (without author data): Baxter et al. (2014, Social Forces). OSF. https://doi.org/10.17605/osf.io/5ywth</t>
         </is>
       </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>@article{mndezchacn2020,
+  author = {Méndez-Chacón, Esteban and Jankowsky, Kristin and Tyner, Andrew H. and Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Parsons, Elan Simon},
+  title = {Reproduction (without author data): Baxter et al. (2014, Social Forces)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/5ywth}
+}</t>
+        </is>
+      </c>
       <c r="D375" t="inlineStr">
         <is>
           <t>Reproduction (without author data): Baxter et al. (2014, Social Forces)</t>
@@ -12367,6 +13170,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., Struhl, M. K., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Chen &amp; van Ours (2018, Demography). OSF. https://doi.org/10.17605/osf.io/kup8x</t>
         </is>
       </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Tyner, Andrew H. and Fox, Nicholas and Struhl, Melissa Kline and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Chen &amp; van Ours (2018, Demography)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/kup8x}
+}</t>
+        </is>
+      </c>
       <c r="D376" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Chen &amp; van Ours (2018, Demography)</t>
@@ -12399,6 +13213,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Grose et al. (2014, American Journal of Political Science). OSF. https://doi.org/10.17605/osf.io/j6c8g</t>
         </is>
       </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Grose et al. (2014, American Journal of Political Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/j6c8g}
+}</t>
+        </is>
+      </c>
       <c r="D377" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Grose et al. (2014, American Journal of Political Science)</t>
@@ -12431,6 +13256,17 @@
           <t>Röer, J. P., Miske, O., Fox, N., Loomas, Z., Luis, B., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Ostermann, T., Michalak, J., &amp; Parsons, E. S. (2020). Reproduction (with author data &amp; code): Hurst &amp; Kavanagh (2017, Evolution and Human Behavior). OSF. https://doi.org/10.17605/osf.io/anfk6</t>
         </is>
       </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>@article{rer2020,
+  author = {Röer, Jan Philipp and Miske, Olivia and Fox, Nicholas and Loomas, Zachary and Luis, Bri and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Ostermann, Thomas and Michalak, Johannes and Parsons, Elan Simon},
+  title = {Reproduction (with author data &amp; code): Hurst &amp; Kavanagh (2017, Evolution and Human Behavior)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/anfk6}
+}</t>
+        </is>
+      </c>
       <c r="D378" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Hurst &amp; Kavanagh (2017, Evolution and Human Behavior)</t>
@@ -12463,6 +13299,17 @@
           <t>Szabelska, A., Tyner, A. H., Loomas, Z., Miske, O., Luis, B., Fox, N., &amp; Hahn, K. (2020). Reproduction (with author data): Nagengast et al. (2014, Journal of Educational Psychology). OSF. https://doi.org/10.17605/osf.io/7p5tw</t>
         </is>
       </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>@article{szabelska2020,
+  author = {Szabelska, Anna and Tyner, Andrew H. and Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Hahn, Krystal},
+  title = {Reproduction (with author data): Nagengast et al. (2014, Journal of Educational Psychology)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/7p5tw}
+}</t>
+        </is>
+      </c>
       <c r="D379" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Nagengast et al. (2014, Journal of Educational Psychology)</t>
@@ -12495,6 +13342,17 @@
           <t>Huntington-Klein, N., Tyner, A. H., Loomas, Z., Miske, O., Fox, N., &amp; Luis, B. (2020). Reproduction (without author data): Horowitz (2018, American Sociological Review). OSF. https://doi.org/10.17605/osf.io/6ye5m</t>
         </is>
       </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>@article{huntingtonklein2020,
+  author = {Huntington-Klein, Nick and Tyner, Andrew H. and Loomas, Zachary and Miske, Olivia and Fox, Nicholas and Luis, Bri},
+  title = {Reproduction (without author data): Horowitz (2018, American Sociological Review)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/6ye5m}
+}</t>
+        </is>
+      </c>
       <c r="D380" t="inlineStr">
         <is>
           <t>Reproduction (without author data): Horowitz (2018, American Sociological Review)</t>
@@ -12527,6 +13385,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Cleave et al. (2013, Experimental Economics). OSF. https://doi.org/10.17605/osf.io/4axu6</t>
         </is>
       </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Cleave et al. (2013, Experimental Economics)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/4axu6}
+}</t>
+        </is>
+      </c>
       <c r="D381" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Cleave et al. (2013, Experimental Economics)</t>
@@ -12559,6 +13428,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Baccara et al. (2014, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/4p892</t>
         </is>
       </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Baccara et al. (2014, American Economic Journal: Applied Economics)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/4p892}
+}</t>
+        </is>
+      </c>
       <c r="D382" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Baccara et al. (2014, American Economic Journal: Applied Economics)</t>
@@ -12591,6 +13471,17 @@
           <t>Gay, V., Tyner, A. H., Luis, B., &amp; Fox, N. (2020). Reproduction (without author data): Mosimann &amp; Pontusson (2017, World Politics). OSF. https://doi.org/10.17605/osf.io/kzpf8</t>
         </is>
       </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>@article{gay2020,
+  author = {Gay, Victor and Tyner, Andrew H. and Luis, Bri and Fox, Nicholas},
+  title = {Reproduction (without author data): Mosimann &amp; Pontusson (2017, World Politics)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/kzpf8}
+}</t>
+        </is>
+      </c>
       <c r="D383" t="inlineStr">
         <is>
           <t>Reproduction (without author data): Mosimann &amp; Pontusson (2017, World Politics)</t>
@@ -12623,6 +13514,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Lee, J. (2021). Reproduction (with author data &amp; code): Sandra &amp; Otto (2018, Cognition). OSF. https://doi.org/10.17605/osf.io/yh25j</t>
         </is>
       </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Lee, Jessica},
+  title = {Reproduction (with author data &amp; code): Sandra &amp; Otto (2018, Cognition)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/yh25j}
+}</t>
+        </is>
+      </c>
       <c r="D384" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Sandra &amp; Otto (2018, Cognition)</t>
@@ -12655,6 +13557,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., Chopik, W. J., &amp; Kołczyńska, M. (2021). Reproduction (with author data &amp; code): Nyhan &amp; Reifler (2015, Journal of Experimental Political Science). OSF. https://doi.org/10.17605/osf.io/5vx27</t>
         </is>
       </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>@article{parsons2021,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Chopik, William J. and Kołczyńska, Marta},
+  title = {Reproduction (with author data &amp; code): Nyhan &amp; Reifler (2015, Journal of Experimental Political Science)},
+  journal = {OSF},
+  year = {2021},
+  doi = {10.17605/osf.io/5vx27}
+}</t>
+        </is>
+      </c>
       <c r="D385" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Nyhan &amp; Reifler (2015, Journal of Experimental Political Science)</t>
@@ -12687,6 +13600,17 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Mushtaq, F. (2022). Reproduction (with author data &amp; code): Rich &amp; Gureckis (2018, Journal of Experimental Psychology: General). OSF. https://doi.org/10.17605/osf.io/u8zk5</t>
         </is>
       </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Mushtaq, Faisal},
+  title = {Reproduction (with author data &amp; code): Rich &amp; Gureckis (2018, Journal of Experimental Psychology: General)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/u8zk5}
+}</t>
+        </is>
+      </c>
       <c r="D386" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Rich &amp; Gureckis (2018, Journal of Experimental Psychology: General)</t>
@@ -12719,6 +13643,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Schmidt, K. (2022). Reproduction (with author data): Savani et al. (2010, Psychological Science). OSF. https://doi.org/10.17605/osf.io/jfxnt</t>
         </is>
       </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Schmidt, Kathleen},
+  title = {Reproduction (with author data): Savani et al. (2010, Psychological Science)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/jfxnt}
+}</t>
+        </is>
+      </c>
       <c r="D387" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Savani et al. (2010, Psychological Science)</t>
@@ -12751,6 +13686,17 @@
           <t>Shaki, S., Miske, O., Loomas, Z., Luis, B., Struhl, M. K., Fox, N., Tyner, A. H., Abatayo, A. L., &amp; Hahn, K. (2020). Reproduction (with author data): Rinaldi et al. (2016, Cognition). OSF. https://doi.org/10.17605/osf.io/8btme</t>
         </is>
       </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>@article{shaki2020,
+  author = {Shaki, Samuel and Miske, Olivia and Loomas, Zachary and Luis, Bri and Struhl, Melissa Kline and Fox, Nicholas and Tyner, Andrew H. and Abatayo, Anna Lou and Hahn, Krystal},
+  title = {Reproduction (with author data): Rinaldi et al. (2016, Cognition)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/8btme}
+}</t>
+        </is>
+      </c>
       <c r="D388" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Rinaldi et al. (2016, Cognition)</t>
@@ -12783,6 +13729,17 @@
           <t>Gereke, J., Field, S., Loomas, Z., Miske, O., Luis, B., Zhang, N., Winter, F., &amp; Kretschmer, D. (2019). Reproduction (without author data): Smith et al. (2016, American Journal of Sociology). OSF. https://doi.org/10.17605/osf.io/nekdp</t>
         </is>
       </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>@article{gereke2019,
+  author = {Gereke, Johanna and Field, Samuel and Loomas, Zachary and Miske, Olivia and Luis, Bri and Zhang, Nan and Winter, Fabian and Kretschmer, David},
+  title = {Reproduction (without author data): Smith et al. (2016, American Journal of Sociology)},
+  journal = {OSF},
+  year = {2019},
+  doi = {10.17605/osf.io/nekdp}
+}</t>
+        </is>
+      </c>
       <c r="D389" t="inlineStr">
         <is>
           <t>Reproduction (without author data): Smith et al. (2016, American Journal of Sociology)</t>
@@ -12815,6 +13772,17 @@
           <t>Chen, J. (., Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Struhl, M. K., Abatayo, A. L., Fox, N., Parsons, E. S., &amp; Hahn, K. (2020). Reproduction (with author data): Goeree et al. (2011, Econometrica). OSF. https://doi.org/10.17605/osf.io/y5uwg</t>
         </is>
       </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>@article{chen2020,
+  author = {Chen, Jingnan (Cecilia) and Miske, Olivia and Loomas, Zachary and Luis, Bri and Tyner, Andrew H. and Struhl, Melissa Kline and Abatayo, Anna Lou and Fox, Nicholas and Parsons, Elan Simon and Hahn, Krystal},
+  title = {Reproduction (with author data): Goeree et al. (2011, Econometrica)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/y5uwg}
+}</t>
+        </is>
+      </c>
       <c r="D390" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Goeree et al. (2011, Econometrica)</t>
@@ -12847,6 +13815,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Izydorczak, K. (2020). Reproduction (with author data &amp; code): Adida et al. (2016, Comparative Political Studies). OSF. https://doi.org/10.17605/osf.io/5k8m4</t>
         </is>
       </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Izydorczak, Kamil},
+  title = {Reproduction (with author data &amp; code): Adida et al. (2016, Comparative Political Studies)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/5k8m4}
+}</t>
+        </is>
+      </c>
       <c r="D391" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Adida et al. (2016, Comparative Political Studies)</t>
@@ -12879,6 +13858,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Talbert, E., Parsons, E. S., &amp; Hahn, K. (2020). Reproduction (with author data &amp; code): Altmann et al. (2012, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/mjb97</t>
         </is>
       </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Talbert, Eli and Parsons, Elan Simon and Hahn, Krystal},
+  title = {Reproduction (with author data &amp; code): Altmann et al. (2012, Journal of Labor Economics)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/mjb97}
+}</t>
+        </is>
+      </c>
       <c r="D392" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Altmann et al. (2012, Journal of Labor Economics)</t>
@@ -12911,6 +13901,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Tyner, A. H., Fox, N., Struhl, M. K., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Baillon et al. (2018, Econometrica). OSF. https://doi.org/10.17605/osf.io/8wf3h</t>
         </is>
       </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Tyner, Andrew H. and Fox, Nicholas and Struhl, Melissa Kline and Abatayo, Anna Lou and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Baillon et al. (2018, Econometrica)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/8wf3h}
+}</t>
+        </is>
+      </c>
       <c r="D393" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Baillon et al. (2018, Econometrica)</t>
@@ -12943,6 +13944,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Akcinaroglu (2012, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/6wfmz</t>
         </is>
       </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Akcinaroglu (2012, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/6wfmz}
+}</t>
+        </is>
+      </c>
       <c r="D394" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Akcinaroglu (2012, Journal of Conflict Resolution)</t>
@@ -12975,6 +13987,16 @@
           <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N. W., Tyner, A. H., &amp; … Silverstein, P. (2026). Reproduction (with author data &amp; code): Luttrell et al. (2016, Journal of Experimental Social Psychology). OSF.</t>
         </is>
       </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>@article{parsons2026,
+  author = {Parsons, E. S. and Miske, O. and Luis, B. and Loomas, Z. and Fox, N. W. and Tyner, A. H. and … Silverstein, P.},
+  title = {Reproduction (with author data &amp; code): Luttrell et al. (2016, Journal of Experimental Social Psychology)},
+  journal = {OSF},
+  year = {2026}
+}</t>
+        </is>
+      </c>
       <c r="D395" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Luttrell et al. (2016, Journal of Experimental Social Psychology)</t>
@@ -13007,6 +14029,16 @@
           <t>Tyner, A. H., Loomas, Z., Miske, O., Luis, B., Breznau, N., Fox, N. W., &amp; Torma, Z. (2026). Reproduction (without author data): Horvat &amp; Evans (2010, European Sociological Review). OSF.</t>
         </is>
       </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>@article{tyner2026,
+  author = {Tyner, A. H. and Loomas, Z. and Miske, O. and Luis, B. and Breznau, N. and Fox, N. W. and Torma, Z.},
+  title = {Reproduction (without author data): Horvat &amp; Evans (2010, European Sociological Review)},
+  journal = {OSF},
+  year = {2026}
+}</t>
+        </is>
+      </c>
       <c r="D396" t="inlineStr">
         <is>
           <t>Reproduction (without author data): Horvat &amp; Evans (2010, European Sociological Review)</t>
@@ -13039,6 +14071,17 @@
           <t>Sonmez, F., Miske, O., Tyner, A. H., Fox, N., Struhl, M. K., Luis, B., &amp; Abatayo, A. L. (2020). Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology). OSF. https://doi.org/10.17605/osf.io/vufm2</t>
         </is>
       </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>@article{sonmez2020,
+  author = {Sonmez, Fatih and Miske, Olivia and Tyner, Andrew H. and Fox, Nicholas and Struhl, Melissa Kline and Luis, Bri and Abatayo, Anna Lou},
+  title = {Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/vufm2}
+}</t>
+        </is>
+      </c>
       <c r="D397" t="inlineStr">
         <is>
           <t>Reproduction (with author data): Ku &amp; Zaroff (2014, Journal of Environmental Psychology)</t>
@@ -13071,6 +14114,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Talbert, E., &amp; Soderberg, C. K. (2020). Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review). OSF. https://doi.org/10.17605/osf.io/m4hqw</t>
         </is>
       </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Talbert, Eli and Soderberg, Courtney K.},
+  title = {Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/m4hqw}
+}</t>
+        </is>
+      </c>
       <c r="D398" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Cohen et al. (2015, American Economic Review)</t>
@@ -13103,6 +14157,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy). OSF. https://doi.org/10.17605/osf.io/37jd4</t>
         </is>
       </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/37jd4}
+}</t>
+        </is>
+      </c>
       <c r="D399" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Clark (2009, Journal of Political Economy)</t>
@@ -13135,6 +14200,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science). OSF. https://doi.org/10.17605/osf.io/g9aqj</t>
         </is>
       </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/g9aqj}
+}</t>
+        </is>
+      </c>
       <c r="D400" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Brown &amp; Kim (2014, Management Science)</t>
@@ -13167,6 +14243,17 @@
           <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica). OSF. https://doi.org/10.17605/osf.io/sv3gb</t>
         </is>
       </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/sv3gb}
+}</t>
+        </is>
+      </c>
       <c r="D401" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): LaFave &amp; Thomas (2016, Econometrica)</t>
@@ -13199,6 +14286,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Tutor, M. (2020). Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics). OSF. https://doi.org/10.17605/osf.io/4n7ef</t>
         </is>
       </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Tutor, Melba},
+  title = {Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/4n7ef}
+}</t>
+        </is>
+      </c>
       <c r="D402" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Lu &amp; Anderson (2015, Journal of Labor Economics)</t>
@@ -13231,6 +14329,17 @@
           <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Talbert, E. (2020). Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution). OSF. https://doi.org/10.17605/osf.io/ysncd</t>
         </is>
       </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Talbert, Eli},
+  title = {Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/ysncd}
+}</t>
+        </is>
+      </c>
       <c r="D403" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): Balcells &amp; Kalyvas (2014, Journal of Conflict Resolution)</t>
@@ -13263,6 +14372,17 @@
           <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Anafinova, S. (2022). Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review). OSF. https://doi.org/10.17605/osf.io/gb46p</t>
         </is>
       </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Anafinova, Saule},
+  title = {Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/gb46p}
+}</t>
+        </is>
+      </c>
       <c r="D404" t="inlineStr">
         <is>
           <t>Reproduction (with author data &amp; code): TERTYTCHNAYA et al. (2018, American Political Science Review)</t>
@@ -13281,6 +14401,866 @@
       <c r="G404" t="inlineStr">
         <is>
           <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/qk9v3</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Antràs_Econometrica_2013_a2Yx - Szabelska - Reproduction (with author data &amp; code) - 28m96. OSF. https://doi.org/10.17605/osf.io/qk9v3</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Antràs_Econometrica_2013_a2Yx - Szabelska - Reproduction (with author data &amp; code) - 28m96},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/qk9v3}
+}</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Antràs_Econometrica_2013_a2Yx - Szabelska - Reproduction (with author data &amp; code) - 28m96</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/7ak4n</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Berry, Z., Miske, O., Loomas, Z., Luis, B., Struhl, M. K., Fox, N., Tyner, A. H., Abatayo, A. L., &amp; Parsons, E. S. (2020). Pastötter_Cognition_2013_EQxa - Berry - Reproduction (with author data) - 3z3k. OSF. https://doi.org/10.17605/osf.io/7ak4n</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>@article{berry2020,
+  author = {Berry, Zachariah and Miske, Olivia and Loomas, Zachary and Luis, Bri and Struhl, Melissa Kline and Fox, Nicholas and Tyner, Andrew H. and Abatayo, Anna Lou and Parsons, Elan Simon},
+  title = {Pastötter_Cognition_2013_EQxa - Berry - Reproduction (with author data) - 3z3k},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/7ak4n}
+}</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Pastötter_Cognition_2013_EQxa - Berry - Reproduction (with author data) - 3z3k</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachariah","family":"Berry","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/zehky</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., Luis, B., &amp; Szabelska, A. (2020). Harper_covid_qKdb - Szabelska - Reproduction (with author data &amp; code) - 1974. OSF. https://doi.org/10.17605/osf.io/zehky</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Luis, Bri and Szabelska, Anna},
+  title = {Harper_covid_qKdb - Szabelska - Reproduction (with author data &amp; code) - 1974},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/zehky}
+}</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Harper_covid_qKdb - Szabelska - Reproduction (with author data &amp; code) - 1974</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/mshda</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Panczak, R., Tyner, A. H., Fox, N., Loomas, Z., Miske, O., &amp; Luis, B. (2020). Siedner_covid_P3NJ - Panczak - Reproduction (without author data) - 1y2. OSF. https://doi.org/10.17605/osf.io/mshda</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>@article{panczak2020,
+  author = {Panczak, Radoslaw and Tyner, Andrew H. and Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri},
+  title = {Siedner_covid_P3NJ - Panczak - Reproduction (without author data) - 1y2},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/mshda}
+}</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Siedner_covid_P3NJ - Panczak - Reproduction (without author data) - 1y2</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>[{"given":"Radoslaw","family":"Panczak","sequence":"first"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/pkwgx</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Freeman, A. L. J., Kerr, J. R., Fox, N., Loomas, Z., Miske, O., &amp; Luis, B. (2020). Rothgerber_covid_BNrd - Freeman - Reproduction (with author data) - 378. OSF. https://doi.org/10.17605/osf.io/pkwgx</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>@article{freeman2020,
+  author = {Freeman, Alexandra L.J. and Kerr, John R. and Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri},
+  title = {Rothgerber_covid_BNrd - Freeman - Reproduction (with author data) - 378},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/pkwgx}
+}</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Rothgerber_covid_BNrd - Freeman - Reproduction (with author data) - 378</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>[{"given":"Alexandra L.J.","family":"Freeman","sequence":"first"},{"given":"John R.","family":"Kerr","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/da26y</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Tyner, A. H., Loomas, Z., Miske, O., Luis, B., Abatayo, A. L., Kołczyńska, M., &amp; Struhl, M. K. (2020). Du_covid_2NAG - Kolczynska - Secondary Data Replication - 41z0. OSF. https://doi.org/10.17605/osf.io/da26y</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>@article{tyner2020,
+  author = {Tyner, Andrew H. and Loomas, Zachary and Miske, Olivia and Luis, Bri and Abatayo, Anna Lou and Kołczyńska, Marta and Struhl, Melissa Kline},
+  title = {Du_covid_2NAG - Kolczynska - Secondary Data Replication - 41z0},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/da26y}
+}</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Du_covid_2NAG - Kolczynska - Secondary Data Replication - 41z0</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>[{"given":"Andrew H.","family":"Tyner","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Marta","family":"Kołczyńska","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/54syu</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Evans, T. R. (2020). Bertin_covid_zk94 - Evans - Reproduction (with author data) - 50z6. OSF. https://doi.org/10.17605/osf.io/54syu</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Evans, Thomas Rhys},
+  title = {Bertin_covid_zk94 - Evans - Reproduction (with author data) - 50z6},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/54syu}
+}</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Bertin_covid_zk94 - Evans - Reproduction (with author data) - 50z6</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Thomas Rhys","family":"Evans","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/w5b24</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., &amp; Evans, T. R. (2020). Plohl_covid_W3vr - Evans - Reproduction (with author data &amp; code) - 538. OSF. https://doi.org/10.17605/osf.io/w5b24</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Evans, Thomas Rhys},
+  title = {Plohl_covid_W3vr - Evans - Reproduction (with author data &amp; code) - 538},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/w5b24}
+}</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Plohl_covid_W3vr - Evans - Reproduction (with author data &amp; code) - 538</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Thomas Rhys","family":"Evans","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/2e5wr</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Fox, N., Loomas, Z., Miske, O., Luis, B., &amp; Szabelska, A. (2020). Bello_Chavolla_covid_Z3mK - Szabelska - Reproduction (with author data &amp; code) - g9z. OSF. https://doi.org/10.17605/osf.io/2e5wr</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>@article{fox2020,
+  author = {Fox, Nicholas and Loomas, Zachary and Miske, Olivia and Luis, Bri and Szabelska, Anna},
+  title = {Bello_Chavolla_covid_Z3mK - Szabelska - Reproduction (with author data &amp; code) - g9z},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/2e5wr}
+}</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Bello_Chavolla_covid_Z3mK - Szabelska - Reproduction (with author data &amp; code) - g9z</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>[{"given":"Nicholas","family":"Fox","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/xrymd</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Szabelska, A. (2020). Rosenfeld_covid_5N2E - Szabelska - Reproduction (with author data &amp; code) - zzz1. OSF. https://doi.org/10.17605/osf.io/xrymd</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Szabelska, Anna},
+  title = {Rosenfeld_covid_5N2E - Szabelska - Reproduction (with author data &amp; code) - zzz1},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/xrymd}
+}</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Rosenfeld_covid_5N2E - Szabelska - Reproduction (with author data &amp; code) - zzz1</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/2uxrt</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Calderón_JournConflictRes_2015_Nv99 - Szabelska - Reproduction (with author data &amp; code) - 6ow1o. OSF. https://doi.org/10.17605/osf.io/2uxrt</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Calderón_JournConflictRes_2015_Nv99 - Szabelska - Reproduction (with author data &amp; code) - 6ow1o},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/2uxrt}
+}</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Calderón_JournConflictRes_2015_Nv99 - Szabelska - Reproduction (with author data &amp; code) - 6ow1o</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/8sae9</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Freeman, A. L. J., Schneider, C. R., Miske, O., Loomas, Z., Luis, B., Fox, N., &amp; Tyner, A. H. (2020). Stanley_covid_b3G4 - Freeman - Reproduction (with author data) - 2z3g. OSF. https://doi.org/10.17605/osf.io/8sae9</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>@article{freeman2020,
+  author = {Freeman, Alexandra L.J. and Schneider, Claudia R. and Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Tyner, Andrew H.},
+  title = {Stanley_covid_b3G4 - Freeman - Reproduction (with author data) - 2z3g},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/8sae9}
+}</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Stanley_covid_b3G4 - Freeman - Reproduction (with author data) - 2z3g</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>[{"given":"Alexandra L.J.","family":"Freeman","sequence":"first"},{"given":"Claudia R.","family":"Schneider","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/rkh2a</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Szabelska, A. (2020). Flesia_covid_P39Z - Szabelska - Reproduction (with author data) - ykg6. OSF. https://doi.org/10.17605/osf.io/rkh2a</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Szabelska, Anna},
+  title = {Flesia_covid_P39Z - Szabelska - Reproduction (with author data) - ykg6},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/rkh2a}
+}</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Flesia_covid_P39Z - Szabelska - Reproduction (with author data) - ykg6</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/2vust</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Chen, J. (., Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Parsons, E. S., &amp; Hahn, K. (2020). Rodriguez-Lara_ExpEco_2012_AgO1 - Chen - Reproduction (with author data) - 9y8y. OSF. https://doi.org/10.17605/osf.io/2vust</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>@article{chen2020,
+  author = {Chen, Jingnan (Cecilia) and Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Parsons, Elan Simon and Hahn, Krystal},
+  title = {Rodriguez-Lara_ExpEco_2012_AgO1 - Chen - Reproduction (with author data) - 9y8y},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/2vust}
+}</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Rodriguez-Lara_ExpEco_2012_AgO1 - Chen - Reproduction (with author data) - 9y8y</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>[{"given":"Jingnan (Cecilia)","family":"Chen","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Elan Simon","family":"Parsons","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/9c5sm</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Talbert, E., &amp; Tyner, A. H. (2020). Pennycook_covid_E32j - Talbert - Reproduction (with author data &amp; code) - 994g. OSF. https://doi.org/10.17605/osf.io/9c5sm</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Talbert, Eli and Tyner, Andrew H.},
+  title = {Pennycook_covid_E32j - Talbert - Reproduction (with author data &amp; code) - 994g},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/9c5sm}
+}</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Pennycook_covid_E32j - Talbert - Reproduction (with author data &amp; code) - 994g</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/r9bdx</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Talbert, E. (2020). Sweeny_covid_2Nzk - Talbert - Reproduction (with author data &amp; code) - 50m6. OSF. https://doi.org/10.17605/osf.io/r9bdx</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Talbert, Eli},
+  title = {Sweeny_covid_2Nzk - Talbert - Reproduction (with author data &amp; code) - 50m6},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/r9bdx}
+}</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Sweeny_covid_2Nzk - Talbert - Reproduction (with author data &amp; code) - 50m6</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Eli","family":"Talbert","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/jvwer</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Miske, O., Loomas, Z., Luis, B., Fox, N., Struhl, M. K., Tyner, A. H., Abatayo, A. L., &amp; Szabelska, A. (2020). Gelfand_covid_R3eV - Szabelska - Reproduction (with author data &amp; code) - zz51. OSF. https://doi.org/10.17605/osf.io/jvwer</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>@article{miske2020,
+  author = {Miske, Olivia and Loomas, Zachary and Luis, Bri and Fox, Nicholas and Struhl, Melissa Kline and Tyner, Andrew H. and Abatayo, Anna Lou and Szabelska, Anna},
+  title = {Gelfand_covid_R3eV - Szabelska - Reproduction (with author data &amp; code) - zz51},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/jvwer}
+}</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Gelfand_covid_R3eV - Szabelska - Reproduction (with author data &amp; code) - zz51</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>[{"given":"Olivia","family":"Miske","sequence":"first"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Melissa Kline","family":"Struhl","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Anna Lou","family":"Abatayo","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/v2yaq</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Loomas, Z., Miske, O., Luis, B., Fox, N., Tyner, A. H., Hahn, K., &amp; Clochard, G. J. (2022). Reproduction (with author data &amp; code): Platt Boustan (2012, American Economic Journal: Applied Economics). OSF. https://doi.org/10.17605/osf.io/v2yaq</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>@article{loomas2022,
+  author = {Loomas, Zachary and Miske, Olivia and Luis, Bri and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Clochard, Gwen-Jiro},
+  title = {Reproduction (with author data &amp; code): Platt Boustan (2012, American Economic Journal: Applied Economics)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/v2yaq}
+}</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): Platt Boustan (2012, American Economic Journal: Applied Economics)</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>[{"given":"Zachary","family":"Loomas","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Gwen-Jiro","family":"Clochard","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/qd3rm</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Parsons, E. S., Miske, O., Luis, B., Loomas, Z., Fox, N., Tyner, A. H., Hahn, K., &amp; Szabelska, A. (2022). Reproduction (with author data &amp; code): ANN SLOCUM et al. (2010, Criminology). OSF. https://doi.org/10.17605/osf.io/qd3rm</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>@article{parsons2022,
+  author = {Parsons, Elan Simon and Miske, Olivia and Luis, Bri and Loomas, Zachary and Fox, Nicholas and Tyner, Andrew H. and Hahn, Krystal and Szabelska, Anna},
+  title = {Reproduction (with author data &amp; code): ANN SLOCUM et al. (2010, Criminology)},
+  journal = {OSF},
+  year = {2022},
+  doi = {10.17605/osf.io/qd3rm}
+}</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Reproduction (with author data &amp; code): ANN SLOCUM et al. (2010, Criminology)</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>[{"given":"Elan Simon","family":"Parsons","sequence":"first"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Nicholas","family":"Fox","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Krystal","family":"Hahn","sequence":"additional"},{"given":"Anna","family":"Szabelska","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>10.17605/osf.io/zfxk9</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Reed, W. R., Coupe, T., Vo, D., Tyner, A. H., Loomas, Z., Miske, O., &amp; Luis, B. (2020). Secondary &amp; Original Data Replication: Bingham Powell (2009, Comparative Political Studies). OSF. https://doi.org/10.17605/osf.io/zfxk9</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>@article{reed2020,
+  author = {Reed, W. Robert and Coupe, Tom and Vo, Diem and Tyner, Andrew H. and Loomas, Zachary and Miske, Olivia and Luis, Bri},
+  title = {Secondary &amp; Original Data Replication: Bingham Powell (2009, Comparative Political Studies)},
+  journal = {OSF},
+  year = {2020},
+  doi = {10.17605/osf.io/zfxk9}
+}</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Secondary &amp; Original Data Replication: Bingham Powell (2009, Comparative Political Studies)</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>[{"given":"W. Robert","family":"Reed","sequence":"first"},{"given":"Tom","family":"Coupe","sequence":"additional"},{"given":"Diem","family":"Vo","sequence":"additional"},{"given":"Andrew H.","family":"Tyner","sequence":"additional"},{"given":"Zachary","family":"Loomas","sequence":"additional"},{"given":"Olivia","family":"Miske","sequence":"additional"},{"given":"Bri","family":"Luis","sequence":"additional"}]</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>OSF</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>2020</t>
         </is>
       </c>
     </row>

</xml_diff>